<commit_message>
Atualização automática: 2026-07-12 00:57 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -80,46 +80,172 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Classificação</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Ativas</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Mobilizadas D-1</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Frota parada</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Alertas</t>
+          <t>11/07/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>Ativas (total)</t>
         </is>
       </c>
       <c r="B2">
         <v>74</v>
       </c>
-      <c r="C2">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ativas - CPTu / VT / SH</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ativas - SEGURANÇA</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ativas - SM</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ativas - SP</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ativas - SP/SM</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ativas - ST | PI | BL  (PI)</t>
+        </is>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Ativas - ST | PI | BL (ST)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 (total)</t>
+        </is>
+      </c>
+      <c r="B10">
         <v>45</v>
       </c>
-      <c r="D2">
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 - SM</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 - SP</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 - SP/SM</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
+        </is>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Frota parada</t>
+        </is>
+      </c>
+      <c r="B16">
         <v>17</v>
       </c>
-      <c r="E2">
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Alertas</t>
+        </is>
+      </c>
+      <c r="B17">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-12 07:50 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -88,6 +88,11 @@
           <t>11/07/2026</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -98,6 +103,9 @@
       <c r="B2">
         <v>74</v>
       </c>
+      <c r="C2">
+        <v>74</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -108,6 +116,9 @@
       <c r="B3">
         <v>4</v>
       </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -118,6 +129,9 @@
       <c r="B4">
         <v>1</v>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -128,6 +142,9 @@
       <c r="B5">
         <v>35</v>
       </c>
+      <c r="C5">
+        <v>35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -138,6 +155,9 @@
       <c r="B6">
         <v>26</v>
       </c>
+      <c r="C6">
+        <v>26</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -148,6 +168,9 @@
       <c r="B7">
         <v>1</v>
       </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -158,6 +181,9 @@
       <c r="B8">
         <v>2</v>
       </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -168,6 +194,9 @@
       <c r="B9">
         <v>5</v>
       </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -178,6 +207,9 @@
       <c r="B10">
         <v>45</v>
       </c>
+      <c r="C10">
+        <v>45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -188,6 +220,9 @@
       <c r="B11">
         <v>25</v>
       </c>
+      <c r="C11">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -198,6 +233,9 @@
       <c r="B12">
         <v>15</v>
       </c>
+      <c r="C12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -208,6 +246,9 @@
       <c r="B13">
         <v>1</v>
       </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -218,6 +259,9 @@
       <c r="B14">
         <v>1</v>
       </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -228,6 +272,9 @@
       <c r="B15">
         <v>3</v>
       </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -238,6 +285,9 @@
       <c r="B16">
         <v>17</v>
       </c>
+      <c r="C16">
+        <v>17</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -246,6 +296,9 @@
         </is>
       </c>
       <c r="B17">
+        <v>34</v>
+      </c>
+      <c r="C17">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore historico.json entries lost by an earlier bad deploy
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -85,6 +85,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>12/07/2026</t>
         </is>
       </c>
@@ -98,6 +103,9 @@
       <c r="B2">
         <v>74</v>
       </c>
+      <c r="C2">
+        <v>74</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -108,6 +116,9 @@
       <c r="B3">
         <v>4</v>
       </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -118,6 +129,9 @@
       <c r="B4">
         <v>1</v>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -128,6 +142,9 @@
       <c r="B5">
         <v>35</v>
       </c>
+      <c r="C5">
+        <v>35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -138,6 +155,9 @@
       <c r="B6">
         <v>26</v>
       </c>
+      <c r="C6">
+        <v>26</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -148,6 +168,9 @@
       <c r="B7">
         <v>1</v>
       </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -158,6 +181,9 @@
       <c r="B8">
         <v>2</v>
       </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -168,6 +194,9 @@
       <c r="B9">
         <v>5</v>
       </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -178,6 +207,9 @@
       <c r="B10">
         <v>45</v>
       </c>
+      <c r="C10">
+        <v>45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -188,6 +220,9 @@
       <c r="B11">
         <v>25</v>
       </c>
+      <c r="C11">
+        <v>25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -198,6 +233,9 @@
       <c r="B12">
         <v>15</v>
       </c>
+      <c r="C12">
+        <v>15</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -208,6 +246,9 @@
       <c r="B13">
         <v>1</v>
       </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -218,6 +259,9 @@
       <c r="B14">
         <v>1</v>
       </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -228,6 +272,9 @@
       <c r="B15">
         <v>3</v>
       </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -238,6 +285,9 @@
       <c r="B16">
         <v>17</v>
       </c>
+      <c r="C16">
+        <v>17</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -246,6 +296,9 @@
         </is>
       </c>
       <c r="B17">
+        <v>34</v>
+      </c>
+      <c r="C17">
         <v>34</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 11:42 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -93,6 +93,11 @@
           <t>12/07/2026</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -106,6 +111,9 @@
       <c r="C2">
         <v>74</v>
       </c>
+      <c r="D2">
+        <v>75</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -119,6 +127,9 @@
       <c r="C3">
         <v>4</v>
       </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -132,6 +143,9 @@
       <c r="C4">
         <v>1</v>
       </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -145,6 +159,9 @@
       <c r="C5">
         <v>35</v>
       </c>
+      <c r="D5">
+        <v>35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -158,6 +175,9 @@
       <c r="C6">
         <v>26</v>
       </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -171,6 +191,9 @@
       <c r="C7">
         <v>1</v>
       </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -184,6 +207,9 @@
       <c r="C8">
         <v>2</v>
       </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -197,6 +223,9 @@
       <c r="C9">
         <v>5</v>
       </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -210,6 +239,9 @@
       <c r="C10">
         <v>45</v>
       </c>
+      <c r="D10">
+        <v>32</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -223,6 +255,9 @@
       <c r="C11">
         <v>25</v>
       </c>
+      <c r="D11">
+        <v>17</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -236,6 +271,9 @@
       <c r="C12">
         <v>15</v>
       </c>
+      <c r="D12">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -249,6 +287,9 @@
       <c r="C13">
         <v>1</v>
       </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -262,6 +303,9 @@
       <c r="C14">
         <v>1</v>
       </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -275,6 +319,9 @@
       <c r="C15">
         <v>3</v>
       </c>
+      <c r="D15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -288,6 +335,9 @@
       <c r="C16">
         <v>17</v>
       </c>
+      <c r="D16">
+        <v>18</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -300,6 +350,9 @@
       </c>
       <c r="C17">
         <v>34</v>
+      </c>
+      <c r="D17">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 18:19 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -112,7 +112,7 @@
         <v>74</v>
       </c>
       <c r="D2">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -240,61 +240,65 @@
         <v>45</v>
       </c>
       <c r="D10">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SM</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>25</v>
-      </c>
-      <c r="C11">
-        <v>25</v>
+          <t>Mobilizadas D-1 - CPTu / VT / SH</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="D11">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP</t>
+          <t>Mobilizadas D-1 - SM</t>
         </is>
       </c>
       <c r="B12">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C12">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D12">
-        <v>11</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP/SM</t>
+          <t>Mobilizadas D-1 - SP</t>
         </is>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
+          <t>Mobilizadas D-1 - SP/SM</t>
         </is>
       </c>
       <c r="B14">
@@ -310,49 +314,65 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
+          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
         </is>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Frota parada</t>
+          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
         </is>
       </c>
       <c r="B16">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C16">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="D16">
-        <v>18</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Frota parada</t>
+        </is>
+      </c>
+      <c r="B17">
+        <v>17</v>
+      </c>
+      <c r="C17">
+        <v>17</v>
+      </c>
+      <c r="D17">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Alertas</t>
         </is>
       </c>
-      <c r="B17">
+      <c r="B18">
         <v>34</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>34</v>
       </c>
-      <c r="D17">
-        <v>35</v>
+      <c r="D18">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 22:41 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -112,7 +112,7 @@
         <v>74</v>
       </c>
       <c r="D2">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3">
@@ -176,7 +176,7 @@
         <v>26</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -224,7 +224,7 @@
         <v>5</v>
       </c>
       <c r="D9">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -372,7 +372,7 @@
         <v>34</v>
       </c>
       <c r="D18">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-14 07:23 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -98,6 +98,11 @@
           <t>13/07/2026</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -114,6 +119,9 @@
       <c r="D2">
         <v>78</v>
       </c>
+      <c r="E2">
+        <v>78</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -130,6 +138,9 @@
       <c r="D3">
         <v>4</v>
       </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -146,6 +157,9 @@
       <c r="D4">
         <v>1</v>
       </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -162,6 +176,9 @@
       <c r="D5">
         <v>35</v>
       </c>
+      <c r="E5">
+        <v>35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -178,6 +195,9 @@
       <c r="D6">
         <v>27</v>
       </c>
+      <c r="E6">
+        <v>27</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -194,6 +214,9 @@
       <c r="D7">
         <v>1</v>
       </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -210,6 +233,9 @@
       <c r="D8">
         <v>2</v>
       </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -226,6 +252,9 @@
       <c r="D9">
         <v>7</v>
       </c>
+      <c r="E9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -242,6 +271,9 @@
       <c r="D10">
         <v>34</v>
       </c>
+      <c r="E10">
+        <v>48</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -262,59 +294,77 @@
       <c r="D11">
         <v>1</v>
       </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SM</t>
-        </is>
-      </c>
-      <c r="B12">
-        <v>25</v>
-      </c>
-      <c r="C12">
-        <v>25</v>
-      </c>
-      <c r="D12">
-        <v>18</v>
+          <t>Mobilizadas D-1 - SEGURANÇA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E12">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP</t>
+          <t>Mobilizadas D-1 - SM</t>
         </is>
       </c>
       <c r="B13">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C13">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D13">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="E13">
+        <v>27</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP/SM</t>
+          <t>Mobilizadas D-1 - SP</t>
         </is>
       </c>
       <c r="B14">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="E14">
+        <v>14</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
+          <t>Mobilizadas D-1 - SP/SM</t>
         </is>
       </c>
       <c r="B15">
@@ -324,54 +374,85 @@
         <v>1</v>
       </c>
       <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
+          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
         </is>
       </c>
       <c r="B16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Frota parada</t>
+          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
         </is>
       </c>
       <c r="B17">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C17">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="D17">
-        <v>18</v>
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Frota parada</t>
+        </is>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
+      <c r="D18">
+        <v>18</v>
+      </c>
+      <c r="E18">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Alertas</t>
         </is>
       </c>
-      <c r="B18">
+      <c r="B19">
         <v>34</v>
       </c>
-      <c r="C18">
+      <c r="C19">
         <v>34</v>
       </c>
-      <c r="D18">
+      <c r="D19">
+        <v>29</v>
+      </c>
+      <c r="E19">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-14 21:32 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -120,7 +120,7 @@
         <v>78</v>
       </c>
       <c r="E2">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -177,7 +177,7 @@
         <v>35</v>
       </c>
       <c r="E5">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-15 06:28 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -103,6 +103,11 @@
           <t>14/07/2026</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -122,6 +127,9 @@
       <c r="E2">
         <v>79</v>
       </c>
+      <c r="F2">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -141,6 +149,9 @@
       <c r="E3">
         <v>4</v>
       </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -160,6 +171,9 @@
       <c r="E4">
         <v>1</v>
       </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -179,6 +193,9 @@
       <c r="E5">
         <v>36</v>
       </c>
+      <c r="F5">
+        <v>36</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -198,6 +215,9 @@
       <c r="E6">
         <v>27</v>
       </c>
+      <c r="F6">
+        <v>27</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -217,6 +237,9 @@
       <c r="E7">
         <v>1</v>
       </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -236,6 +259,9 @@
       <c r="E8">
         <v>2</v>
       </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -255,6 +281,9 @@
       <c r="E9">
         <v>7</v>
       </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -274,6 +303,9 @@
       <c r="E10">
         <v>48</v>
       </c>
+      <c r="F10">
+        <v>46</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -297,6 +329,9 @@
       <c r="E11">
         <v>1</v>
       </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -322,6 +357,9 @@
       <c r="E12">
         <v>1</v>
       </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -341,6 +379,9 @@
       <c r="E13">
         <v>27</v>
       </c>
+      <c r="F13">
+        <v>25</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -360,6 +401,9 @@
       <c r="E14">
         <v>14</v>
       </c>
+      <c r="F14">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -379,6 +423,9 @@
       <c r="E15">
         <v>1</v>
       </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -398,6 +445,9 @@
       <c r="E16">
         <v>1</v>
       </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -417,6 +467,9 @@
       <c r="E17">
         <v>3</v>
       </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -436,6 +489,9 @@
       <c r="E18">
         <v>20</v>
       </c>
+      <c r="F18">
+        <v>19</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -454,6 +510,9 @@
       </c>
       <c r="E19">
         <v>32</v>
+      </c>
+      <c r="F19">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-15 17:59 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -304,7 +304,7 @@
         <v>48</v>
       </c>
       <c r="F10">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
@@ -380,7 +380,7 @@
         <v>27</v>
       </c>
       <c r="F13">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-15 21:32 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -128,7 +128,7 @@
         <v>79</v>
       </c>
       <c r="F2">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -172,7 +172,7 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -194,7 +194,7 @@
         <v>36</v>
       </c>
       <c r="F5">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -216,7 +216,7 @@
         <v>27</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -304,7 +304,7 @@
         <v>48</v>
       </c>
       <c r="F10">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -402,7 +402,7 @@
         <v>14</v>
       </c>
       <c r="F14">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -512,7 +512,7 @@
         <v>32</v>
       </c>
       <c r="F19">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-16 13:06 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -108,6 +108,11 @@
           <t>15/07/2026</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -130,6 +135,9 @@
       <c r="F2">
         <v>84</v>
       </c>
+      <c r="G2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -152,6 +160,9 @@
       <c r="F3">
         <v>4</v>
       </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -174,6 +185,9 @@
       <c r="F4">
         <v>2</v>
       </c>
+      <c r="G4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -196,6 +210,9 @@
       <c r="F5">
         <v>38</v>
       </c>
+      <c r="G5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -218,6 +235,9 @@
       <c r="F6">
         <v>30</v>
       </c>
+      <c r="G6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -240,6 +260,9 @@
       <c r="F7">
         <v>1</v>
       </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -262,6 +285,9 @@
       <c r="F8">
         <v>2</v>
       </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -284,6 +310,9 @@
       <c r="F9">
         <v>7</v>
       </c>
+      <c r="G9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -306,6 +335,9 @@
       <c r="F10">
         <v>46</v>
       </c>
+      <c r="G10">
+        <v>37</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -332,6 +364,11 @@
       <c r="F11">
         <v>1</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -360,6 +397,11 @@
       <c r="F12">
         <v>1</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -382,6 +424,9 @@
       <c r="F13">
         <v>26</v>
       </c>
+      <c r="G13">
+        <v>18</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -404,6 +449,9 @@
       <c r="F14">
         <v>14</v>
       </c>
+      <c r="G14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -426,6 +474,9 @@
       <c r="F15">
         <v>1</v>
       </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -448,6 +499,9 @@
       <c r="F16">
         <v>1</v>
       </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -470,6 +524,9 @@
       <c r="F17">
         <v>2</v>
       </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -492,6 +549,9 @@
       <c r="F18">
         <v>19</v>
       </c>
+      <c r="G18">
+        <v>21</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -512,6 +572,9 @@
         <v>32</v>
       </c>
       <c r="F19">
+        <v>29</v>
+      </c>
+      <c r="G19">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-16 17:56 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -336,7 +336,7 @@
         <v>46</v>
       </c>
       <c r="G10">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -425,7 +425,7 @@
         <v>26</v>
       </c>
       <c r="G13">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14">
@@ -575,7 +575,7 @@
         <v>29</v>
       </c>
       <c r="G19">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-17 06:27 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -113,6 +113,11 @@
           <t>16/07/2026</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -138,6 +143,9 @@
       <c r="G2">
         <v>84</v>
       </c>
+      <c r="H2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -163,6 +171,9 @@
       <c r="G3">
         <v>4</v>
       </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -188,6 +199,9 @@
       <c r="G4">
         <v>2</v>
       </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -213,6 +227,9 @@
       <c r="G5">
         <v>38</v>
       </c>
+      <c r="H5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -238,6 +255,9 @@
       <c r="G6">
         <v>30</v>
       </c>
+      <c r="H6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -263,6 +283,9 @@
       <c r="G7">
         <v>1</v>
       </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -288,6 +311,9 @@
       <c r="G8">
         <v>2</v>
       </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -313,6 +339,9 @@
       <c r="G9">
         <v>7</v>
       </c>
+      <c r="H9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -338,6 +367,9 @@
       <c r="G10">
         <v>36</v>
       </c>
+      <c r="H10">
+        <v>43</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -369,6 +401,11 @@
           <t/>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -402,6 +439,9 @@
           <t/>
         </is>
       </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -427,6 +467,9 @@
       <c r="G13">
         <v>17</v>
       </c>
+      <c r="H13">
+        <v>26</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -452,6 +495,9 @@
       <c r="G14">
         <v>13</v>
       </c>
+      <c r="H14">
+        <v>11</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -477,6 +523,9 @@
       <c r="G15">
         <v>1</v>
       </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -502,6 +551,9 @@
       <c r="G16">
         <v>1</v>
       </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -527,6 +579,9 @@
       <c r="G17">
         <v>4</v>
       </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -552,6 +607,9 @@
       <c r="G18">
         <v>21</v>
       </c>
+      <c r="H18">
+        <v>20</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -575,6 +633,9 @@
         <v>29</v>
       </c>
       <c r="G19">
+        <v>28</v>
+      </c>
+      <c r="H19">
         <v>28</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-18 05:54 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -118,6 +118,11 @@
           <t>17/07/2026</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>18/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -146,6 +151,9 @@
       <c r="H2">
         <v>84</v>
       </c>
+      <c r="I2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -174,6 +182,9 @@
       <c r="H3">
         <v>4</v>
       </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -202,6 +213,9 @@
       <c r="H4">
         <v>2</v>
       </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -230,6 +244,9 @@
       <c r="H5">
         <v>38</v>
       </c>
+      <c r="I5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -258,6 +275,9 @@
       <c r="H6">
         <v>30</v>
       </c>
+      <c r="I6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -286,6 +306,9 @@
       <c r="H7">
         <v>1</v>
       </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -314,6 +337,9 @@
       <c r="H8">
         <v>2</v>
       </c>
+      <c r="I8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -342,6 +368,9 @@
       <c r="H9">
         <v>7</v>
       </c>
+      <c r="I9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -370,6 +399,9 @@
       <c r="H10">
         <v>43</v>
       </c>
+      <c r="I10">
+        <v>46</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -406,6 +438,11 @@
           <t/>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -442,6 +479,9 @@
       <c r="H12">
         <v>1</v>
       </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -470,6 +510,9 @@
       <c r="H13">
         <v>26</v>
       </c>
+      <c r="I13">
+        <v>26</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -498,6 +541,9 @@
       <c r="H14">
         <v>11</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -526,6 +572,9 @@
       <c r="H15">
         <v>1</v>
       </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -554,6 +603,9 @@
       <c r="H16">
         <v>2</v>
       </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -582,6 +634,9 @@
       <c r="H17">
         <v>2</v>
       </c>
+      <c r="I17">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -610,6 +665,9 @@
       <c r="H18">
         <v>20</v>
       </c>
+      <c r="I18">
+        <v>22</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -636,6 +694,9 @@
         <v>28</v>
       </c>
       <c r="H19">
+        <v>29</v>
+      </c>
+      <c r="I19">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-18 15:30 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -400,7 +400,7 @@
         <v>43</v>
       </c>
       <c r="I10">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
@@ -511,7 +511,7 @@
         <v>26</v>
       </c>
       <c r="I13">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -542,7 +542,7 @@
         <v>11</v>
       </c>
       <c r="I14">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-18 18:40 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -400,7 +400,7 @@
         <v>43</v>
       </c>
       <c r="I10">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
@@ -542,7 +542,7 @@
         <v>11</v>
       </c>
       <c r="I14">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-19 07:49 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -123,6 +123,11 @@
           <t>18/07/2026</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>19/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -154,6 +159,9 @@
       <c r="I2">
         <v>84</v>
       </c>
+      <c r="J2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -185,6 +193,9 @@
       <c r="I3">
         <v>4</v>
       </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -216,6 +227,9 @@
       <c r="I4">
         <v>2</v>
       </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -247,6 +261,9 @@
       <c r="I5">
         <v>38</v>
       </c>
+      <c r="J5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -278,6 +295,9 @@
       <c r="I6">
         <v>30</v>
       </c>
+      <c r="J6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -309,6 +329,9 @@
       <c r="I7">
         <v>1</v>
       </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -340,6 +363,9 @@
       <c r="I8">
         <v>2</v>
       </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -371,6 +397,9 @@
       <c r="I9">
         <v>7</v>
       </c>
+      <c r="J9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -402,6 +431,9 @@
       <c r="I10">
         <v>47</v>
       </c>
+      <c r="J10">
+        <v>49</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -443,6 +475,9 @@
           <t/>
         </is>
       </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -482,6 +517,9 @@
       <c r="I12">
         <v>1</v>
       </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -513,6 +551,9 @@
       <c r="I13">
         <v>27</v>
       </c>
+      <c r="J13">
+        <v>29</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -544,6 +585,9 @@
       <c r="I14">
         <v>13</v>
       </c>
+      <c r="J14">
+        <v>12</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -575,6 +619,9 @@
       <c r="I15">
         <v>1</v>
       </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -606,6 +653,9 @@
       <c r="I16">
         <v>1</v>
       </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -637,6 +687,9 @@
       <c r="I17">
         <v>4</v>
       </c>
+      <c r="J17">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -668,6 +721,9 @@
       <c r="I18">
         <v>22</v>
       </c>
+      <c r="J18">
+        <v>21</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -697,6 +753,9 @@
         <v>29</v>
       </c>
       <c r="I19">
+        <v>29</v>
+      </c>
+      <c r="J19">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-20 10:32 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -128,6 +128,11 @@
           <t>19/07/2026</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -162,6 +167,9 @@
       <c r="J2">
         <v>84</v>
       </c>
+      <c r="K2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -196,6 +204,9 @@
       <c r="J3">
         <v>4</v>
       </c>
+      <c r="K3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -230,6 +241,9 @@
       <c r="J4">
         <v>2</v>
       </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -264,6 +278,9 @@
       <c r="J5">
         <v>38</v>
       </c>
+      <c r="K5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -298,6 +315,9 @@
       <c r="J6">
         <v>30</v>
       </c>
+      <c r="K6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -332,6 +352,9 @@
       <c r="J7">
         <v>1</v>
       </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -366,6 +389,9 @@
       <c r="J8">
         <v>2</v>
       </c>
+      <c r="K8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -400,6 +426,9 @@
       <c r="J9">
         <v>7</v>
       </c>
+      <c r="K9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -434,6 +463,9 @@
       <c r="J10">
         <v>49</v>
       </c>
+      <c r="K10">
+        <v>43</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -478,6 +510,9 @@
       <c r="J11">
         <v>1</v>
       </c>
+      <c r="K11">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -520,6 +555,11 @@
       <c r="J12">
         <v>1</v>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -554,6 +594,9 @@
       <c r="J13">
         <v>29</v>
       </c>
+      <c r="K13">
+        <v>23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -588,6 +631,9 @@
       <c r="J14">
         <v>12</v>
       </c>
+      <c r="K14">
+        <v>14</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -622,6 +668,11 @@
       <c r="J15">
         <v>1</v>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -656,6 +707,9 @@
       <c r="J16">
         <v>1</v>
       </c>
+      <c r="K16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -690,6 +744,9 @@
       <c r="J17">
         <v>4</v>
       </c>
+      <c r="K17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -724,6 +781,9 @@
       <c r="J18">
         <v>21</v>
       </c>
+      <c r="K18">
+        <v>22</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -757,6 +817,9 @@
       </c>
       <c r="J19">
         <v>29</v>
+      </c>
+      <c r="K19">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-20 17:07 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -168,7 +168,7 @@
         <v>84</v>
       </c>
       <c r="K2">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -205,7 +205,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -279,7 +279,7 @@
         <v>38</v>
       </c>
       <c r="K5">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
@@ -464,7 +464,7 @@
         <v>49</v>
       </c>
       <c r="K10">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11">
@@ -595,7 +595,7 @@
         <v>29</v>
       </c>
       <c r="K13">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
@@ -632,7 +632,7 @@
         <v>12</v>
       </c>
       <c r="K14">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -819,7 +819,7 @@
         <v>29</v>
       </c>
       <c r="K19">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-20 21:49 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -168,7 +168,7 @@
         <v>84</v>
       </c>
       <c r="K2">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -279,7 +279,7 @@
         <v>38</v>
       </c>
       <c r="K5">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -316,7 +316,7 @@
         <v>30</v>
       </c>
       <c r="K6">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -352,8 +352,10 @@
       <c r="J7">
         <v>1</v>
       </c>
-      <c r="K7">
-        <v>1</v>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -464,7 +466,7 @@
         <v>49</v>
       </c>
       <c r="K10">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
@@ -595,7 +597,7 @@
         <v>29</v>
       </c>
       <c r="K13">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14">
@@ -819,7 +821,7 @@
         <v>29</v>
       </c>
       <c r="K19">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-21 07:42 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -133,6 +133,11 @@
           <t>20/07/2026</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>21/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -170,6 +175,9 @@
       <c r="K2">
         <v>85</v>
       </c>
+      <c r="L2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -207,6 +215,9 @@
       <c r="K3">
         <v>5</v>
       </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -244,6 +255,9 @@
       <c r="K4">
         <v>2</v>
       </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -281,6 +295,9 @@
       <c r="K5">
         <v>37</v>
       </c>
+      <c r="L5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -318,6 +335,9 @@
       <c r="K6">
         <v>32</v>
       </c>
+      <c r="L6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -357,6 +377,11 @@
           <t/>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -394,6 +419,9 @@
       <c r="K8">
         <v>2</v>
       </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -431,6 +459,9 @@
       <c r="K9">
         <v>7</v>
       </c>
+      <c r="L9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -468,6 +499,9 @@
       <c r="K10">
         <v>42</v>
       </c>
+      <c r="L10">
+        <v>38</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -515,6 +549,9 @@
       <c r="K11">
         <v>2</v>
       </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -562,6 +599,11 @@
           <t/>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -599,6 +641,9 @@
       <c r="K13">
         <v>23</v>
       </c>
+      <c r="L13">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -636,6 +681,9 @@
       <c r="K14">
         <v>13</v>
       </c>
+      <c r="L14">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -675,6 +723,11 @@
           <t/>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -712,6 +765,9 @@
       <c r="K16">
         <v>2</v>
       </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -749,6 +805,9 @@
       <c r="K17">
         <v>2</v>
       </c>
+      <c r="L17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -786,6 +845,9 @@
       <c r="K18">
         <v>22</v>
       </c>
+      <c r="L18">
+        <v>26</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -822,6 +884,9 @@
       </c>
       <c r="K19">
         <v>27</v>
+      </c>
+      <c r="L19">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-21 13:04 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -176,7 +176,7 @@
         <v>85</v>
       </c>
       <c r="L2">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -846,7 +846,7 @@
         <v>22</v>
       </c>
       <c r="L18">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-22 09:17 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -138,6 +138,11 @@
           <t>21/07/2026</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>22/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -178,6 +183,9 @@
       <c r="L2">
         <v>85</v>
       </c>
+      <c r="M2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -218,6 +226,9 @@
       <c r="L3">
         <v>5</v>
       </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -258,6 +269,9 @@
       <c r="L4">
         <v>2</v>
       </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -298,6 +312,9 @@
       <c r="L5">
         <v>37</v>
       </c>
+      <c r="M5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -338,6 +355,9 @@
       <c r="L6">
         <v>32</v>
       </c>
+      <c r="M6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -382,6 +402,11 @@
           <t/>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -422,6 +447,9 @@
       <c r="L8">
         <v>2</v>
       </c>
+      <c r="M8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -462,6 +490,9 @@
       <c r="L9">
         <v>7</v>
       </c>
+      <c r="M9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -502,6 +533,9 @@
       <c r="L10">
         <v>38</v>
       </c>
+      <c r="M10">
+        <v>41</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -552,6 +586,9 @@
       <c r="L11">
         <v>1</v>
       </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -604,6 +641,11 @@
           <t/>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -644,6 +686,9 @@
       <c r="L13">
         <v>24</v>
       </c>
+      <c r="M13">
+        <v>22</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -684,6 +729,9 @@
       <c r="L14">
         <v>10</v>
       </c>
+      <c r="M14">
+        <v>14</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -728,6 +776,11 @@
           <t/>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -768,6 +821,9 @@
       <c r="L16">
         <v>1</v>
       </c>
+      <c r="M16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -808,6 +864,9 @@
       <c r="L17">
         <v>2</v>
       </c>
+      <c r="M17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -848,6 +907,9 @@
       <c r="L18">
         <v>27</v>
       </c>
+      <c r="M18">
+        <v>25</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -887,6 +949,9 @@
       </c>
       <c r="L19">
         <v>29</v>
+      </c>
+      <c r="M19">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-23 07:44 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -143,6 +143,11 @@
           <t>22/07/2026</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -186,6 +191,9 @@
       <c r="M2">
         <v>86</v>
       </c>
+      <c r="N2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -229,6 +237,9 @@
       <c r="M3">
         <v>5</v>
       </c>
+      <c r="N3">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -272,6 +283,9 @@
       <c r="M4">
         <v>2</v>
       </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -315,6 +329,9 @@
       <c r="M5">
         <v>37</v>
       </c>
+      <c r="N5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -358,6 +375,9 @@
       <c r="M6">
         <v>32</v>
       </c>
+      <c r="N6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -407,6 +427,11 @@
           <t/>
         </is>
       </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -450,6 +475,9 @@
       <c r="M8">
         <v>2</v>
       </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -493,6 +521,9 @@
       <c r="M9">
         <v>7</v>
       </c>
+      <c r="N9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -536,6 +567,9 @@
       <c r="M10">
         <v>41</v>
       </c>
+      <c r="N10">
+        <v>38</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -589,6 +623,9 @@
       <c r="M11">
         <v>1</v>
       </c>
+      <c r="N11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -646,6 +683,9 @@
           <t/>
         </is>
       </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -689,6 +729,9 @@
       <c r="M13">
         <v>22</v>
       </c>
+      <c r="N13">
+        <v>22</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -732,6 +775,9 @@
       <c r="M14">
         <v>14</v>
       </c>
+      <c r="N14">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -781,6 +827,11 @@
           <t/>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -824,6 +875,9 @@
       <c r="M16">
         <v>2</v>
       </c>
+      <c r="N16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -867,6 +921,9 @@
       <c r="M17">
         <v>2</v>
       </c>
+      <c r="N17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -910,6 +967,9 @@
       <c r="M18">
         <v>25</v>
       </c>
+      <c r="N18">
+        <v>25</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -952,6 +1012,9 @@
       </c>
       <c r="M19">
         <v>27</v>
+      </c>
+      <c r="N19">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-23 13:13 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -238,7 +238,7 @@
         <v>5</v>
       </c>
       <c r="N3">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -476,7 +476,7 @@
         <v>2</v>
       </c>
       <c r="N8">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -568,7 +568,7 @@
         <v>41</v>
       </c>
       <c r="N10">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11">
@@ -876,7 +876,7 @@
         <v>2</v>
       </c>
       <c r="N16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -922,7 +922,7 @@
         <v>2</v>
       </c>
       <c r="N17">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -968,7 +968,7 @@
         <v>25</v>
       </c>
       <c r="N18">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-24 08:00 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -148,6 +148,11 @@
           <t>23/07/2026</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -194,6 +199,9 @@
       <c r="N2">
         <v>85</v>
       </c>
+      <c r="O2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -240,6 +248,9 @@
       <c r="N3">
         <v>4</v>
       </c>
+      <c r="O3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -286,6 +297,9 @@
       <c r="N4">
         <v>2</v>
       </c>
+      <c r="O4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -332,6 +346,9 @@
       <c r="N5">
         <v>37</v>
       </c>
+      <c r="O5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -378,6 +395,9 @@
       <c r="N6">
         <v>32</v>
       </c>
+      <c r="O6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -432,6 +452,11 @@
           <t/>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -478,6 +503,9 @@
       <c r="N8">
         <v>3</v>
       </c>
+      <c r="O8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -524,6 +552,9 @@
       <c r="N9">
         <v>7</v>
       </c>
+      <c r="O9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -570,6 +601,9 @@
       <c r="N10">
         <v>40</v>
       </c>
+      <c r="O10">
+        <v>44</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -626,6 +660,9 @@
       <c r="N11">
         <v>1</v>
       </c>
+      <c r="O11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -686,6 +723,9 @@
       <c r="N12">
         <v>1</v>
       </c>
+      <c r="O12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -732,6 +772,9 @@
       <c r="N13">
         <v>22</v>
       </c>
+      <c r="O13">
+        <v>23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -778,6 +821,9 @@
       <c r="N14">
         <v>10</v>
       </c>
+      <c r="O14">
+        <v>14</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -832,6 +878,11 @@
           <t/>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -878,6 +929,9 @@
       <c r="N16">
         <v>3</v>
       </c>
+      <c r="O16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -924,6 +978,9 @@
       <c r="N17">
         <v>3</v>
       </c>
+      <c r="O17">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -970,6 +1027,9 @@
       <c r="N18">
         <v>26</v>
       </c>
+      <c r="O18">
+        <v>23</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1014,6 +1074,9 @@
         <v>27</v>
       </c>
       <c r="N19">
+        <v>23</v>
+      </c>
+      <c r="O19">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-24 15:18 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -602,7 +602,7 @@
         <v>40</v>
       </c>
       <c r="O10">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11">
@@ -773,7 +773,7 @@
         <v>22</v>
       </c>
       <c r="O13">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14">
@@ -822,7 +822,7 @@
         <v>10</v>
       </c>
       <c r="O14">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -1028,7 +1028,7 @@
         <v>26</v>
       </c>
       <c r="O18">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -1077,7 +1077,7 @@
         <v>23</v>
       </c>
       <c r="O19">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-25 06:30 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -153,6 +153,11 @@
           <t>24/07/2026</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -202,6 +207,9 @@
       <c r="O2">
         <v>85</v>
       </c>
+      <c r="P2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -251,6 +259,9 @@
       <c r="O3">
         <v>4</v>
       </c>
+      <c r="P3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -300,6 +311,9 @@
       <c r="O4">
         <v>2</v>
       </c>
+      <c r="P4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -349,6 +363,9 @@
       <c r="O5">
         <v>37</v>
       </c>
+      <c r="P5">
+        <v>36</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -398,6 +415,9 @@
       <c r="O6">
         <v>32</v>
       </c>
+      <c r="P6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -457,6 +477,11 @@
           <t/>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -506,6 +531,9 @@
       <c r="O8">
         <v>3</v>
       </c>
+      <c r="P8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -555,6 +583,9 @@
       <c r="O9">
         <v>7</v>
       </c>
+      <c r="P9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -604,6 +635,9 @@
       <c r="O10">
         <v>46</v>
       </c>
+      <c r="P10">
+        <v>45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -663,6 +697,9 @@
       <c r="O11">
         <v>1</v>
       </c>
+      <c r="P11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -726,6 +763,9 @@
       <c r="O12">
         <v>1</v>
       </c>
+      <c r="P12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -775,6 +815,9 @@
       <c r="O13">
         <v>24</v>
       </c>
+      <c r="P13">
+        <v>23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -824,6 +867,9 @@
       <c r="O14">
         <v>15</v>
       </c>
+      <c r="P14">
+        <v>16</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -883,6 +929,11 @@
           <t/>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -932,6 +983,9 @@
       <c r="O16">
         <v>2</v>
       </c>
+      <c r="P16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -981,6 +1035,11 @@
       <c r="O17">
         <v>3</v>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1030,6 +1089,9 @@
       <c r="O18">
         <v>24</v>
       </c>
+      <c r="P18">
+        <v>23</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1077,6 +1139,9 @@
         <v>23</v>
       </c>
       <c r="O19">
+        <v>21</v>
+      </c>
+      <c r="P19">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-26 07:45 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -158,6 +158,11 @@
           <t>25/07/2026</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -210,6 +215,9 @@
       <c r="P2">
         <v>84</v>
       </c>
+      <c r="Q2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -262,6 +270,9 @@
       <c r="P3">
         <v>4</v>
       </c>
+      <c r="Q3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -314,6 +325,9 @@
       <c r="P4">
         <v>2</v>
       </c>
+      <c r="Q4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -366,6 +380,9 @@
       <c r="P5">
         <v>36</v>
       </c>
+      <c r="Q5">
+        <v>36</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -418,6 +435,9 @@
       <c r="P6">
         <v>32</v>
       </c>
+      <c r="Q6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -482,6 +502,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -534,6 +559,9 @@
       <c r="P8">
         <v>3</v>
       </c>
+      <c r="Q8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -586,6 +614,9 @@
       <c r="P9">
         <v>7</v>
       </c>
+      <c r="Q9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -638,6 +669,9 @@
       <c r="P10">
         <v>45</v>
       </c>
+      <c r="Q10">
+        <v>46</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -700,6 +734,9 @@
       <c r="P11">
         <v>1</v>
       </c>
+      <c r="Q11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -766,6 +803,9 @@
       <c r="P12">
         <v>2</v>
       </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -818,6 +858,9 @@
       <c r="P13">
         <v>23</v>
       </c>
+      <c r="Q13">
+        <v>23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -870,6 +913,9 @@
       <c r="P14">
         <v>16</v>
       </c>
+      <c r="Q14">
+        <v>19</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -934,6 +980,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -986,6 +1037,9 @@
       <c r="P16">
         <v>3</v>
       </c>
+      <c r="Q16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1040,6 +1094,11 @@
           <t/>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1092,6 +1151,9 @@
       <c r="P18">
         <v>23</v>
       </c>
+      <c r="Q18">
+        <v>24</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1142,6 +1204,9 @@
         <v>21</v>
       </c>
       <c r="P19">
+        <v>21</v>
+      </c>
+      <c r="Q19">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-26 15:44 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -670,7 +670,7 @@
         <v>45</v>
       </c>
       <c r="Q10">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11">
@@ -859,7 +859,7 @@
         <v>23</v>
       </c>
       <c r="Q13">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 10:55 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -163,6 +163,11 @@
           <t>26/07/2026</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -218,6 +223,9 @@
       <c r="Q2">
         <v>84</v>
       </c>
+      <c r="R2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -273,6 +281,9 @@
       <c r="Q3">
         <v>4</v>
       </c>
+      <c r="R3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -328,6 +339,9 @@
       <c r="Q4">
         <v>2</v>
       </c>
+      <c r="R4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -383,6 +397,9 @@
       <c r="Q5">
         <v>36</v>
       </c>
+      <c r="R5">
+        <v>36</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -438,6 +455,9 @@
       <c r="Q6">
         <v>32</v>
       </c>
+      <c r="R6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -507,6 +527,11 @@
           <t/>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -562,6 +587,9 @@
       <c r="Q8">
         <v>3</v>
       </c>
+      <c r="R8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -617,6 +645,9 @@
       <c r="Q9">
         <v>7</v>
       </c>
+      <c r="R9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -672,6 +703,9 @@
       <c r="Q10">
         <v>45</v>
       </c>
+      <c r="R10">
+        <v>46</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -737,6 +771,11 @@
       <c r="Q11">
         <v>1</v>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -806,6 +845,9 @@
       <c r="Q12">
         <v>1</v>
       </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -861,6 +903,9 @@
       <c r="Q13">
         <v>22</v>
       </c>
+      <c r="R13">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -916,6 +961,9 @@
       <c r="Q14">
         <v>19</v>
       </c>
+      <c r="R14">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -985,6 +1033,11 @@
           <t/>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1040,6 +1093,9 @@
       <c r="Q16">
         <v>2</v>
       </c>
+      <c r="R16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1099,6 +1155,9 @@
           <t/>
         </is>
       </c>
+      <c r="R17">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1154,6 +1213,9 @@
       <c r="Q18">
         <v>24</v>
       </c>
+      <c r="R18">
+        <v>24</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1208,6 +1270,9 @@
       </c>
       <c r="Q19">
         <v>21</v>
+      </c>
+      <c r="R19">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 17:59 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1214,7 +1214,7 @@
         <v>24</v>
       </c>
       <c r="R18">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">
@@ -1272,7 +1272,7 @@
         <v>21</v>
       </c>
       <c r="R19">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 21:48 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -224,7 +224,7 @@
         <v>84</v>
       </c>
       <c r="R2">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -398,7 +398,7 @@
         <v>36</v>
       </c>
       <c r="R5">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -704,7 +704,7 @@
         <v>45</v>
       </c>
       <c r="R10">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
@@ -904,7 +904,7 @@
         <v>22</v>
       </c>
       <c r="R13">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
@@ -1094,7 +1094,7 @@
         <v>2</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1214,7 +1214,7 @@
         <v>24</v>
       </c>
       <c r="R18">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 07:47 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -168,6 +168,11 @@
           <t>27/07/2026</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -226,6 +231,9 @@
       <c r="R2">
         <v>86</v>
       </c>
+      <c r="S2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -284,6 +292,9 @@
       <c r="R3">
         <v>4</v>
       </c>
+      <c r="S3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -342,6 +353,9 @@
       <c r="R4">
         <v>2</v>
       </c>
+      <c r="S4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -400,6 +414,9 @@
       <c r="R5">
         <v>37</v>
       </c>
+      <c r="S5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -458,6 +475,9 @@
       <c r="R6">
         <v>33</v>
       </c>
+      <c r="S6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -532,6 +552,11 @@
           <t/>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -590,6 +615,9 @@
       <c r="R8">
         <v>3</v>
       </c>
+      <c r="S8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -648,6 +676,9 @@
       <c r="R9">
         <v>7</v>
       </c>
+      <c r="S9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -706,6 +737,9 @@
       <c r="R10">
         <v>48</v>
       </c>
+      <c r="S10">
+        <v>53</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -776,6 +810,9 @@
           <t/>
         </is>
       </c>
+      <c r="S11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -848,6 +885,9 @@
       <c r="R12">
         <v>1</v>
       </c>
+      <c r="S12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -906,6 +946,9 @@
       <c r="R13">
         <v>21</v>
       </c>
+      <c r="S13">
+        <v>23</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -964,6 +1007,9 @@
       <c r="R14">
         <v>20</v>
       </c>
+      <c r="S14">
+        <v>24</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1038,6 +1084,11 @@
           <t/>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1096,6 +1147,9 @@
       <c r="R16">
         <v>3</v>
       </c>
+      <c r="S16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1158,6 +1212,9 @@
       <c r="R17">
         <v>3</v>
       </c>
+      <c r="S17">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1216,6 +1273,9 @@
       <c r="R18">
         <v>25</v>
       </c>
+      <c r="S18">
+        <v>26</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1272,6 +1332,9 @@
         <v>21</v>
       </c>
       <c r="R19">
+        <v>23</v>
+      </c>
+      <c r="S19">
         <v>23</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 15:54 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -947,7 +947,7 @@
         <v>21</v>
       </c>
       <c r="S13">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
@@ -1148,7 +1148,7 @@
         <v>3</v>
       </c>
       <c r="S16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1274,7 +1274,7 @@
         <v>25</v>
       </c>
       <c r="S18">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -1335,7 +1335,7 @@
         <v>23</v>
       </c>
       <c r="S19">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-29 08:02 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -173,6 +173,11 @@
           <t>28/07/2026</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -234,6 +239,9 @@
       <c r="S2">
         <v>86</v>
       </c>
+      <c r="T2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -295,6 +303,9 @@
       <c r="S3">
         <v>4</v>
       </c>
+      <c r="T3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -356,6 +367,9 @@
       <c r="S4">
         <v>2</v>
       </c>
+      <c r="T4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -417,6 +431,9 @@
       <c r="S5">
         <v>37</v>
       </c>
+      <c r="T5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -478,6 +495,9 @@
       <c r="S6">
         <v>33</v>
       </c>
+      <c r="T6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -557,6 +577,11 @@
           <t/>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -618,6 +643,9 @@
       <c r="S8">
         <v>3</v>
       </c>
+      <c r="T8">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -679,6 +707,9 @@
       <c r="S9">
         <v>7</v>
       </c>
+      <c r="T9">
+        <v>7</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -740,6 +771,9 @@
       <c r="S10">
         <v>53</v>
       </c>
+      <c r="T10">
+        <v>60</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -813,6 +847,9 @@
       <c r="S11">
         <v>1</v>
       </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -888,6 +925,11 @@
       <c r="S12">
         <v>1</v>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -949,6 +991,9 @@
       <c r="S13">
         <v>22</v>
       </c>
+      <c r="T13">
+        <v>24</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1010,6 +1055,9 @@
       <c r="S14">
         <v>24</v>
       </c>
+      <c r="T14">
+        <v>29</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1089,6 +1137,11 @@
           <t/>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1150,6 +1203,9 @@
       <c r="S16">
         <v>2</v>
       </c>
+      <c r="T16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1215,6 +1271,9 @@
       <c r="S17">
         <v>3</v>
       </c>
+      <c r="T17">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1276,6 +1335,9 @@
       <c r="S18">
         <v>25</v>
       </c>
+      <c r="T18">
+        <v>24</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1335,6 +1397,9 @@
         <v>23</v>
       </c>
       <c r="S19">
+        <v>26</v>
+      </c>
+      <c r="T19">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-29 15:58 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -643,218 +643,244 @@
       <c r="S8">
         <v>3</v>
       </c>
-      <c r="T8">
-        <v>3</v>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ativas - ST | PI | BL (ST)</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>5</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="D9">
-        <v>7</v>
-      </c>
-      <c r="E9">
-        <v>7</v>
-      </c>
-      <c r="F9">
-        <v>7</v>
-      </c>
-      <c r="G9">
-        <v>7</v>
-      </c>
-      <c r="H9">
-        <v>7</v>
-      </c>
-      <c r="I9">
-        <v>7</v>
-      </c>
-      <c r="J9">
-        <v>7</v>
-      </c>
-      <c r="K9">
-        <v>7</v>
-      </c>
-      <c r="L9">
-        <v>7</v>
-      </c>
-      <c r="M9">
-        <v>7</v>
-      </c>
-      <c r="N9">
-        <v>7</v>
-      </c>
-      <c r="O9">
-        <v>7</v>
-      </c>
-      <c r="P9">
-        <v>7</v>
-      </c>
-      <c r="Q9">
-        <v>7</v>
-      </c>
-      <c r="R9">
-        <v>7</v>
-      </c>
-      <c r="S9">
-        <v>7</v>
+          <t>Ativas - ST | PI | BL (PI)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="T9">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 (total)</t>
+          <t>Ativas - ST | PI | BL (ST)</t>
         </is>
       </c>
       <c r="B10">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C10">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="D10">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="F10">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="G10">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="H10">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="I10">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="J10">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="K10">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="L10">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="M10">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="N10">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="O10">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="P10">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="Q10">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="R10">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="S10">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="T10">
-        <v>60</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - CPTu / VT / SH</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+          <t>Mobilizadas D-1 (total)</t>
+        </is>
+      </c>
+      <c r="B11">
+        <v>45</v>
+      </c>
+      <c r="C11">
+        <v>45</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>46</v>
+      </c>
+      <c r="G11">
+        <v>36</v>
+      </c>
+      <c r="H11">
+        <v>43</v>
+      </c>
+      <c r="I11">
+        <v>47</v>
       </c>
       <c r="J11">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="N11">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="O11">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="P11">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="Q11">
-        <v>1</v>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>45</v>
+      </c>
+      <c r="R11">
+        <v>48</v>
       </c>
       <c r="S11">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SEGURANÇA</t>
+          <t>Mobilizadas D-1 - CPTu / VT / SH</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -867,10 +893,8 @@
           <t/>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="D12">
+        <v>1</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -883,29 +907,27 @@
           <t/>
         </is>
       </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
-      <c r="I12">
-        <v>1</v>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="J12">
         <v>1</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="K12">
+        <v>2</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
       </c>
       <c r="N12">
         <v>1</v>
@@ -914,239 +936,235 @@
         <v>1</v>
       </c>
       <c r="P12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q12">
         <v>1</v>
       </c>
-      <c r="R12">
-        <v>1</v>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="S12">
         <v>1</v>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="T12">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SM</t>
-        </is>
-      </c>
-      <c r="B13">
-        <v>25</v>
-      </c>
-      <c r="C13">
-        <v>25</v>
-      </c>
-      <c r="D13">
-        <v>18</v>
+          <t>Mobilizadas D-1 - SEGURANÇA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="E13">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>26</v>
-      </c>
-      <c r="G13">
-        <v>17</v>
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="H13">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="J13">
-        <v>29</v>
-      </c>
-      <c r="K13">
-        <v>23</v>
-      </c>
-      <c r="L13">
-        <v>24</v>
-      </c>
-      <c r="M13">
-        <v>22</v>
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="N13">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="O13">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="P13">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="Q13">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="R13">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="S13">
-        <v>22</v>
-      </c>
-      <c r="T13">
-        <v>24</v>
+        <v>1</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP</t>
+          <t>Mobilizadas D-1 - SM</t>
         </is>
       </c>
       <c r="B14">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C14">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D14">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E14">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F14">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G14">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I14">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="J14">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="K14">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="L14">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="M14">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="N14">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="O14">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="P14">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="Q14">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="R14">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S14">
+        <v>22</v>
+      </c>
+      <c r="T14">
         <v>24</v>
-      </c>
-      <c r="T14">
-        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - SP/SM</t>
+          <t>Mobilizadas D-1 - SP</t>
         </is>
       </c>
       <c r="B15">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="H15">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="K15">
+        <v>13</v>
+      </c>
+      <c r="L15">
+        <v>10</v>
+      </c>
+      <c r="M15">
+        <v>14</v>
+      </c>
+      <c r="N15">
+        <v>10</v>
+      </c>
+      <c r="O15">
+        <v>15</v>
+      </c>
+      <c r="P15">
+        <v>16</v>
+      </c>
+      <c r="Q15">
+        <v>19</v>
+      </c>
+      <c r="R15">
+        <v>20</v>
+      </c>
+      <c r="S15">
+        <v>24</v>
+      </c>
+      <c r="T15">
+        <v>30</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
+          <t>Mobilizadas D-1 - SP/SM</t>
         </is>
       </c>
       <c r="B16">
@@ -1168,7 +1186,7 @@
         <v>1</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -1176,75 +1194,95 @@
       <c r="J16">
         <v>1</v>
       </c>
-      <c r="K16">
-        <v>2</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16">
-        <v>2</v>
-      </c>
-      <c r="N16">
-        <v>3</v>
-      </c>
-      <c r="O16">
-        <v>2</v>
-      </c>
-      <c r="P16">
-        <v>3</v>
-      </c>
-      <c r="Q16">
-        <v>2</v>
-      </c>
-      <c r="R16">
-        <v>3</v>
-      </c>
-      <c r="S16">
-        <v>2</v>
-      </c>
-      <c r="T16">
-        <v>3</v>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
+          <t>Mobilizadas D-1 - ST | PI | BL  (PI)</t>
         </is>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H17">
         <v>2</v>
       </c>
       <c r="I17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K17">
         <v>2</v>
       </c>
       <c r="L17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17">
         <v>2</v>
@@ -1253,153 +1291,319 @@
         <v>3</v>
       </c>
       <c r="O17">
-        <v>3</v>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="P17">
+        <v>3</v>
+      </c>
+      <c r="Q17">
+        <v>2</v>
       </c>
       <c r="R17">
         <v>3</v>
       </c>
       <c r="S17">
-        <v>3</v>
-      </c>
-      <c r="T17">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Frota parada</t>
-        </is>
-      </c>
-      <c r="B18">
-        <v>17</v>
-      </c>
-      <c r="C18">
-        <v>17</v>
-      </c>
-      <c r="D18">
-        <v>18</v>
-      </c>
-      <c r="E18">
-        <v>20</v>
-      </c>
-      <c r="F18">
-        <v>19</v>
-      </c>
-      <c r="G18">
-        <v>21</v>
-      </c>
-      <c r="H18">
-        <v>20</v>
-      </c>
-      <c r="I18">
-        <v>22</v>
-      </c>
-      <c r="J18">
-        <v>21</v>
-      </c>
-      <c r="K18">
-        <v>22</v>
-      </c>
-      <c r="L18">
-        <v>27</v>
-      </c>
-      <c r="M18">
-        <v>25</v>
-      </c>
-      <c r="N18">
-        <v>26</v>
-      </c>
-      <c r="O18">
-        <v>24</v>
-      </c>
-      <c r="P18">
-        <v>23</v>
-      </c>
-      <c r="Q18">
-        <v>24</v>
-      </c>
-      <c r="R18">
-        <v>25</v>
-      </c>
-      <c r="S18">
-        <v>25</v>
+          <t>Mobilizadas D-1 - ST | PI | BL (PI)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="T18">
-        <v>24</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Mobilizadas D-1 - ST | PI | BL (ST)</t>
+        </is>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>4</v>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+      <c r="I19">
+        <v>4</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+      <c r="K19">
+        <v>2</v>
+      </c>
+      <c r="L19">
+        <v>2</v>
+      </c>
+      <c r="M19">
+        <v>2</v>
+      </c>
+      <c r="N19">
+        <v>3</v>
+      </c>
+      <c r="O19">
+        <v>3</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R19">
+        <v>3</v>
+      </c>
+      <c r="S19">
+        <v>3</v>
+      </c>
+      <c r="T19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Frota parada</t>
+        </is>
+      </c>
+      <c r="B20">
+        <v>17</v>
+      </c>
+      <c r="C20">
+        <v>17</v>
+      </c>
+      <c r="D20">
+        <v>18</v>
+      </c>
+      <c r="E20">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <v>19</v>
+      </c>
+      <c r="G20">
+        <v>21</v>
+      </c>
+      <c r="H20">
+        <v>20</v>
+      </c>
+      <c r="I20">
+        <v>22</v>
+      </c>
+      <c r="J20">
+        <v>21</v>
+      </c>
+      <c r="K20">
+        <v>22</v>
+      </c>
+      <c r="L20">
+        <v>27</v>
+      </c>
+      <c r="M20">
+        <v>25</v>
+      </c>
+      <c r="N20">
+        <v>26</v>
+      </c>
+      <c r="O20">
+        <v>24</v>
+      </c>
+      <c r="P20">
+        <v>23</v>
+      </c>
+      <c r="Q20">
+        <v>24</v>
+      </c>
+      <c r="R20">
+        <v>25</v>
+      </c>
+      <c r="S20">
+        <v>25</v>
+      </c>
+      <c r="T20">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Alertas</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B21">
         <v>34</v>
       </c>
-      <c r="C19">
+      <c r="C21">
         <v>34</v>
       </c>
-      <c r="D19">
+      <c r="D21">
         <v>29</v>
       </c>
-      <c r="E19">
+      <c r="E21">
         <v>32</v>
       </c>
-      <c r="F19">
+      <c r="F21">
         <v>29</v>
       </c>
-      <c r="G19">
+      <c r="G21">
         <v>28</v>
       </c>
-      <c r="H19">
+      <c r="H21">
         <v>29</v>
       </c>
-      <c r="I19">
+      <c r="I21">
         <v>29</v>
       </c>
-      <c r="J19">
+      <c r="J21">
         <v>29</v>
       </c>
-      <c r="K19">
+      <c r="K21">
         <v>27</v>
       </c>
-      <c r="L19">
+      <c r="L21">
         <v>29</v>
       </c>
-      <c r="M19">
+      <c r="M21">
         <v>27</v>
       </c>
-      <c r="N19">
+      <c r="N21">
         <v>23</v>
       </c>
-      <c r="O19">
+      <c r="O21">
         <v>21</v>
       </c>
-      <c r="P19">
+      <c r="P21">
         <v>21</v>
       </c>
-      <c r="Q19">
+      <c r="Q21">
         <v>21</v>
       </c>
-      <c r="R19">
+      <c r="R21">
         <v>23</v>
       </c>
-      <c r="S19">
+      <c r="S21">
         <v>26</v>
       </c>
-      <c r="T19">
+      <c r="T21">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-30 07:42 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -178,6 +178,11 @@
           <t>29/07/2026</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -242,6 +247,9 @@
       <c r="T2">
         <v>86</v>
       </c>
+      <c r="U2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -306,6 +314,9 @@
       <c r="T3">
         <v>4</v>
       </c>
+      <c r="U3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -370,6 +381,9 @@
       <c r="T4">
         <v>2</v>
       </c>
+      <c r="U4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -434,6 +448,9 @@
       <c r="T5">
         <v>37</v>
       </c>
+      <c r="U5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -498,6 +515,9 @@
       <c r="T6">
         <v>33</v>
       </c>
+      <c r="U6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -582,6 +602,11 @@
           <t/>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -648,6 +673,11 @@
           <t/>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -748,6 +778,9 @@
       <c r="T9">
         <v>3</v>
       </c>
+      <c r="U9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -812,6 +845,9 @@
       <c r="T10">
         <v>7</v>
       </c>
+      <c r="U10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -876,6 +912,9 @@
       <c r="T11">
         <v>62</v>
       </c>
+      <c r="U11">
+        <v>60</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -952,6 +991,9 @@
       <c r="T12">
         <v>2</v>
       </c>
+      <c r="U12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1032,6 +1074,11 @@
           <t/>
         </is>
       </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1096,6 +1143,9 @@
       <c r="T14">
         <v>24</v>
       </c>
+      <c r="U14">
+        <v>23</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1160,6 +1210,9 @@
       <c r="T15">
         <v>30</v>
       </c>
+      <c r="U15">
+        <v>29</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1244,6 +1297,11 @@
           <t/>
         </is>
       </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1310,6 +1368,11 @@
           <t/>
         </is>
       </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1410,6 +1473,9 @@
       <c r="T18">
         <v>3</v>
       </c>
+      <c r="U18">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1478,6 +1544,9 @@
       <c r="T19">
         <v>3</v>
       </c>
+      <c r="U19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1542,6 +1611,9 @@
       <c r="T20">
         <v>24</v>
       </c>
+      <c r="U20">
+        <v>24</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1604,6 +1676,9 @@
         <v>26</v>
       </c>
       <c r="T21">
+        <v>26</v>
+      </c>
+      <c r="U21">
         <v>26</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-30 18:58 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -248,7 +248,7 @@
         <v>86</v>
       </c>
       <c r="U2">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="U9">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -913,7 +913,7 @@
         <v>62</v>
       </c>
       <c r="U11">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12">
@@ -1474,7 +1474,7 @@
         <v>3</v>
       </c>
       <c r="U18">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1679,7 +1679,7 @@
         <v>26</v>
       </c>
       <c r="U21">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-31 10:03 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -183,6 +183,11 @@
           <t>30/07/2026</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -250,6 +255,9 @@
       <c r="U2">
         <v>84</v>
       </c>
+      <c r="V2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -317,6 +325,9 @@
       <c r="U3">
         <v>4</v>
       </c>
+      <c r="V3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -384,6 +395,9 @@
       <c r="U4">
         <v>2</v>
       </c>
+      <c r="V4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -451,6 +465,9 @@
       <c r="U5">
         <v>37</v>
       </c>
+      <c r="V5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -518,6 +535,9 @@
       <c r="U6">
         <v>32</v>
       </c>
+      <c r="V6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -607,6 +627,11 @@
           <t/>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -678,6 +703,11 @@
           <t/>
         </is>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -781,6 +811,9 @@
       <c r="U9">
         <v>2</v>
       </c>
+      <c r="V9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -848,6 +881,9 @@
       <c r="U10">
         <v>7</v>
       </c>
+      <c r="V10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,6 +951,9 @@
       <c r="U11">
         <v>59</v>
       </c>
+      <c r="V11">
+        <v>55</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -994,6 +1033,11 @@
       <c r="U12">
         <v>2</v>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1079,6 +1123,9 @@
           <t/>
         </is>
       </c>
+      <c r="V13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1146,6 +1193,9 @@
       <c r="U14">
         <v>23</v>
       </c>
+      <c r="V14">
+        <v>22</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1213,6 +1263,9 @@
       <c r="U15">
         <v>29</v>
       </c>
+      <c r="V15">
+        <v>30</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1302,6 +1355,11 @@
           <t/>
         </is>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1373,6 +1431,11 @@
           <t/>
         </is>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1476,6 +1539,9 @@
       <c r="U18">
         <v>2</v>
       </c>
+      <c r="V18">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1547,6 +1613,11 @@
       <c r="U19">
         <v>3</v>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1614,6 +1685,9 @@
       <c r="U20">
         <v>24</v>
       </c>
+      <c r="V20">
+        <v>24</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1679,6 +1753,9 @@
         <v>26</v>
       </c>
       <c r="U21">
+        <v>25</v>
+      </c>
+      <c r="V21">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-31 17:11 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -256,7 +256,7 @@
         <v>84</v>
       </c>
       <c r="V2">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         <v>32</v>
       </c>
       <c r="V6">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -1686,7 +1686,7 @@
         <v>24</v>
       </c>
       <c r="V20">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-01 07:20 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -188,6 +188,11 @@
           <t>31/07/2026</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -258,6 +263,9 @@
       <c r="V2">
         <v>85</v>
       </c>
+      <c r="W2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -328,6 +336,9 @@
       <c r="V3">
         <v>4</v>
       </c>
+      <c r="W3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -398,6 +409,9 @@
       <c r="V4">
         <v>2</v>
       </c>
+      <c r="W4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -468,6 +482,9 @@
       <c r="V5">
         <v>37</v>
       </c>
+      <c r="W5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -538,6 +555,9 @@
       <c r="V6">
         <v>33</v>
       </c>
+      <c r="W6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -632,6 +652,11 @@
           <t/>
         </is>
       </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -708,6 +733,11 @@
           <t/>
         </is>
       </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -814,6 +844,9 @@
       <c r="V9">
         <v>2</v>
       </c>
+      <c r="W9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -884,6 +917,9 @@
       <c r="V10">
         <v>7</v>
       </c>
+      <c r="W10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -954,6 +990,9 @@
       <c r="V11">
         <v>55</v>
       </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1038,6 +1077,11 @@
           <t/>
         </is>
       </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1126,6 +1170,11 @@
       <c r="V13">
         <v>1</v>
       </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1196,6 +1245,11 @@
       <c r="V14">
         <v>22</v>
       </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1266,6 +1320,11 @@
       <c r="V15">
         <v>30</v>
       </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1360,6 +1419,11 @@
           <t/>
         </is>
       </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1436,6 +1500,11 @@
           <t/>
         </is>
       </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1542,6 +1611,11 @@
       <c r="V18">
         <v>2</v>
       </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1618,6 +1692,11 @@
           <t/>
         </is>
       </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1688,6 +1767,9 @@
       <c r="V20">
         <v>25</v>
       </c>
+      <c r="W20">
+        <v>14</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1757,6 +1839,9 @@
       </c>
       <c r="V21">
         <v>23</v>
+      </c>
+      <c r="W21">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-02 07:39 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -193,6 +193,11 @@
           <t>01/08/2026</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>02/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -266,6 +271,9 @@
       <c r="W2">
         <v>85</v>
       </c>
+      <c r="X2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -339,6 +347,9 @@
       <c r="W3">
         <v>4</v>
       </c>
+      <c r="X3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -412,6 +423,9 @@
       <c r="W4">
         <v>2</v>
       </c>
+      <c r="X4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -485,6 +499,9 @@
       <c r="W5">
         <v>37</v>
       </c>
+      <c r="X5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -558,6 +575,9 @@
       <c r="W6">
         <v>33</v>
       </c>
+      <c r="X6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -657,6 +677,11 @@
           <t/>
         </is>
       </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -738,6 +763,11 @@
           <t/>
         </is>
       </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -847,6 +877,9 @@
       <c r="W9">
         <v>2</v>
       </c>
+      <c r="X9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -920,6 +953,9 @@
       <c r="W10">
         <v>7</v>
       </c>
+      <c r="X10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -993,6 +1029,9 @@
       <c r="W11">
         <v>0</v>
       </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1082,6 +1121,11 @@
           <t/>
         </is>
       </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1175,6 +1219,11 @@
           <t/>
         </is>
       </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1250,6 +1299,11 @@
           <t/>
         </is>
       </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1325,6 +1379,11 @@
           <t/>
         </is>
       </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1424,6 +1483,11 @@
           <t/>
         </is>
       </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1505,6 +1569,11 @@
           <t/>
         </is>
       </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1616,6 +1685,11 @@
           <t/>
         </is>
       </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1697,6 +1771,11 @@
           <t/>
         </is>
       </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1770,6 +1849,9 @@
       <c r="W20">
         <v>14</v>
       </c>
+      <c r="X20">
+        <v>26</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1841,6 +1923,9 @@
         <v>23</v>
       </c>
       <c r="W21">
+        <v>27</v>
+      </c>
+      <c r="X21">
         <v>27</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-02 14:53 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -1121,10 +1121,8 @@
           <t/>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X12">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1219,10 +1217,8 @@
           <t/>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X13">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1299,10 +1295,8 @@
           <t/>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X14">
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -1379,10 +1373,8 @@
           <t/>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X15">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -1685,10 +1677,8 @@
           <t/>
         </is>
       </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X18">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1771,10 +1761,8 @@
           <t/>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="X19">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1850,7 +1838,7 @@
         <v>14</v>
       </c>
       <c r="X20">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-03 01:23 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -1296,7 +1296,7 @@
         </is>
       </c>
       <c r="X14">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="X15">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="X19">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1914,7 +1914,7 @@
         <v>27</v>
       </c>
       <c r="X21">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-03 05:25 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -198,6 +198,11 @@
           <t>02/08/2026</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -274,6 +279,9 @@
       <c r="X2">
         <v>85</v>
       </c>
+      <c r="Y2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -350,6 +358,9 @@
       <c r="X3">
         <v>4</v>
       </c>
+      <c r="Y3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -426,6 +437,9 @@
       <c r="X4">
         <v>2</v>
       </c>
+      <c r="Y4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -502,6 +516,9 @@
       <c r="X5">
         <v>37</v>
       </c>
+      <c r="Y5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -578,6 +595,9 @@
       <c r="X6">
         <v>33</v>
       </c>
+      <c r="Y6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -682,6 +702,11 @@
           <t/>
         </is>
       </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -768,6 +793,11 @@
           <t/>
         </is>
       </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -880,6 +910,9 @@
       <c r="X9">
         <v>2</v>
       </c>
+      <c r="Y9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -956,6 +989,9 @@
       <c r="X10">
         <v>7</v>
       </c>
+      <c r="Y10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1032,6 +1068,9 @@
       <c r="X11">
         <v>46</v>
       </c>
+      <c r="Y11">
+        <v>46</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1124,6 +1163,9 @@
       <c r="X12">
         <v>2</v>
       </c>
+      <c r="Y12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1220,6 +1262,9 @@
       <c r="X13">
         <v>1</v>
       </c>
+      <c r="Y13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1298,6 +1343,9 @@
       <c r="X14">
         <v>13</v>
       </c>
+      <c r="Y14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1376,6 +1424,9 @@
       <c r="X15">
         <v>28</v>
       </c>
+      <c r="Y15">
+        <v>28</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1480,6 +1531,11 @@
           <t/>
         </is>
       </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1566,6 +1622,11 @@
           <t/>
         </is>
       </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1680,6 +1741,9 @@
       <c r="X18">
         <v>1</v>
       </c>
+      <c r="Y18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1764,6 +1828,9 @@
       <c r="X19">
         <v>1</v>
       </c>
+      <c r="Y19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1840,6 +1907,9 @@
       <c r="X20">
         <v>29</v>
       </c>
+      <c r="Y20">
+        <v>29</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1914,6 +1984,9 @@
         <v>27</v>
       </c>
       <c r="X21">
+        <v>24</v>
+      </c>
+      <c r="Y21">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-03 19:13 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1069,7 +1069,7 @@
         <v>46</v>
       </c>
       <c r="Y11">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -1344,7 +1344,7 @@
         <v>13</v>
       </c>
       <c r="Y14">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15">
@@ -1425,7 +1425,7 @@
         <v>28</v>
       </c>
       <c r="Y15">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -1987,7 +1987,7 @@
         <v>24</v>
       </c>
       <c r="Y21">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-04 01:13 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1069,7 +1069,7 @@
         <v>46</v>
       </c>
       <c r="Y11">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -1344,7 +1344,7 @@
         <v>13</v>
       </c>
       <c r="Y14">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -1425,7 +1425,7 @@
         <v>28</v>
       </c>
       <c r="Y15">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -1742,7 +1742,7 @@
         <v>1</v>
       </c>
       <c r="Y18">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1829,7 +1829,7 @@
         <v>1</v>
       </c>
       <c r="Y19">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -1908,7 +1908,7 @@
         <v>29</v>
       </c>
       <c r="Y20">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
@@ -1987,7 +1987,7 @@
         <v>24</v>
       </c>
       <c r="Y21">
-        <v>22</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-04 04:51 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -203,6 +203,11 @@
           <t>03/08/2026</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>04/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -282,6 +287,9 @@
       <c r="Y2">
         <v>85</v>
       </c>
+      <c r="Z2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -361,6 +369,9 @@
       <c r="Y3">
         <v>4</v>
       </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -440,6 +451,9 @@
       <c r="Y4">
         <v>2</v>
       </c>
+      <c r="Z4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -519,6 +533,9 @@
       <c r="Y5">
         <v>37</v>
       </c>
+      <c r="Z5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -598,6 +615,9 @@
       <c r="Y6">
         <v>33</v>
       </c>
+      <c r="Z6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,6 +727,11 @@
           <t/>
         </is>
       </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -798,6 +823,11 @@
           <t/>
         </is>
       </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -913,6 +943,9 @@
       <c r="Y9">
         <v>2</v>
       </c>
+      <c r="Z9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -992,6 +1025,9 @@
       <c r="Y10">
         <v>7</v>
       </c>
+      <c r="Z10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1071,6 +1107,9 @@
       <c r="Y11">
         <v>50</v>
       </c>
+      <c r="Z11">
+        <v>50</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1166,6 +1205,9 @@
       <c r="Y12">
         <v>2</v>
       </c>
+      <c r="Z12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1265,6 +1307,9 @@
       <c r="Y13">
         <v>1</v>
       </c>
+      <c r="Z13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1346,6 +1391,9 @@
       <c r="Y14">
         <v>17</v>
       </c>
+      <c r="Z14">
+        <v>17</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1427,6 +1475,9 @@
       <c r="Y15">
         <v>25</v>
       </c>
+      <c r="Z15">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1536,6 +1587,11 @@
           <t/>
         </is>
       </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1627,6 +1683,11 @@
           <t/>
         </is>
       </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1744,6 +1805,9 @@
       <c r="Y18">
         <v>2</v>
       </c>
+      <c r="Z18">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1831,6 +1895,9 @@
       <c r="Y19">
         <v>3</v>
       </c>
+      <c r="Z19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1910,6 +1977,9 @@
       <c r="Y20">
         <v>32</v>
       </c>
+      <c r="Z20">
+        <v>32</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1987,6 +2057,9 @@
         <v>24</v>
       </c>
       <c r="Y21">
+        <v>89</v>
+      </c>
+      <c r="Z21">
         <v>89</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-04 11:52 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -288,7 +288,7 @@
         <v>85</v>
       </c>
       <c r="Z2">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -616,7 +616,7 @@
         <v>33</v>
       </c>
       <c r="Z6">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -2060,7 +2060,7 @@
         <v>89</v>
       </c>
       <c r="Z21">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-05 01:15 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1108,7 +1108,7 @@
         <v>50</v>
       </c>
       <c r="Z11">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -1206,7 +1206,7 @@
         <v>2</v>
       </c>
       <c r="Z12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1392,7 +1392,7 @@
         <v>17</v>
       </c>
       <c r="Z14">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -1476,7 +1476,7 @@
         <v>25</v>
       </c>
       <c r="Z15">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16">
@@ -1806,7 +1806,7 @@
         <v>2</v>
       </c>
       <c r="Z18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1896,7 +1896,7 @@
         <v>3</v>
       </c>
       <c r="Z19">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1978,7 +1978,7 @@
         <v>32</v>
       </c>
       <c r="Z20">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
@@ -2060,7 +2060,7 @@
         <v>89</v>
       </c>
       <c r="Z21">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-05 04:51 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -208,6 +208,11 @@
           <t>04/08/2026</t>
         </is>
       </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -290,6 +295,9 @@
       <c r="Z2">
         <v>84</v>
       </c>
+      <c r="AA2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -372,6 +380,9 @@
       <c r="Z3">
         <v>4</v>
       </c>
+      <c r="AA3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -454,6 +465,9 @@
       <c r="Z4">
         <v>2</v>
       </c>
+      <c r="AA4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -536,6 +550,9 @@
       <c r="Z5">
         <v>37</v>
       </c>
+      <c r="AA5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -618,6 +635,9 @@
       <c r="Z6">
         <v>32</v>
       </c>
+      <c r="AA6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,6 +752,11 @@
           <t/>
         </is>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -828,6 +853,11 @@
           <t/>
         </is>
       </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -946,6 +976,9 @@
       <c r="Z9">
         <v>2</v>
       </c>
+      <c r="AA9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1028,6 +1061,9 @@
       <c r="Z10">
         <v>7</v>
       </c>
+      <c r="AA10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1110,6 +1146,9 @@
       <c r="Z11">
         <v>51</v>
       </c>
+      <c r="AA11">
+        <v>51</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1208,6 +1247,9 @@
       <c r="Z12">
         <v>1</v>
       </c>
+      <c r="AA12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1310,6 +1352,9 @@
       <c r="Z13">
         <v>1</v>
       </c>
+      <c r="AA13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1394,6 +1439,9 @@
       <c r="Z14">
         <v>18</v>
       </c>
+      <c r="AA14">
+        <v>18</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1478,6 +1526,9 @@
       <c r="Z15">
         <v>29</v>
       </c>
+      <c r="AA15">
+        <v>29</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1592,6 +1643,11 @@
           <t/>
         </is>
       </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1688,6 +1744,11 @@
           <t/>
         </is>
       </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1808,6 +1869,9 @@
       <c r="Z18">
         <v>1</v>
       </c>
+      <c r="AA18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1898,6 +1962,9 @@
       <c r="Z19">
         <v>1</v>
       </c>
+      <c r="AA19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1980,6 +2047,9 @@
       <c r="Z20">
         <v>30</v>
       </c>
+      <c r="AA20">
+        <v>30</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2060,6 +2130,9 @@
         <v>89</v>
       </c>
       <c r="Z21">
+        <v>86</v>
+      </c>
+      <c r="AA21">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-05 20:52 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -296,7 +296,7 @@
         <v>84</v>
       </c>
       <c r="AA2">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -636,7 +636,7 @@
         <v>32</v>
       </c>
       <c r="AA6">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -2133,7 +2133,7 @@
         <v>86</v>
       </c>
       <c r="AA21">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-06 01:12 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1147,7 +1147,7 @@
         <v>51</v>
       </c>
       <c r="AA11">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -1440,7 +1440,7 @@
         <v>18</v>
       </c>
       <c r="AA14">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -2048,7 +2048,7 @@
         <v>30</v>
       </c>
       <c r="AA20">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-06 04:51 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -213,6 +213,11 @@
           <t>05/08/2026</t>
         </is>
       </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>06/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -298,6 +303,9 @@
       <c r="AA2">
         <v>83</v>
       </c>
+      <c r="AB2">
+        <v>83</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -383,6 +391,9 @@
       <c r="AA3">
         <v>4</v>
       </c>
+      <c r="AB3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -468,6 +479,9 @@
       <c r="AA4">
         <v>2</v>
       </c>
+      <c r="AB4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -553,6 +567,9 @@
       <c r="AA5">
         <v>37</v>
       </c>
+      <c r="AB5">
+        <v>37</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -638,6 +655,9 @@
       <c r="AA6">
         <v>31</v>
       </c>
+      <c r="AB6">
+        <v>31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -757,6 +777,11 @@
           <t/>
         </is>
       </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -858,6 +883,11 @@
           <t/>
         </is>
       </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -979,6 +1009,9 @@
       <c r="AA9">
         <v>2</v>
       </c>
+      <c r="AB9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1064,6 +1097,9 @@
       <c r="AA10">
         <v>7</v>
       </c>
+      <c r="AB10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1149,6 +1185,9 @@
       <c r="AA11">
         <v>49</v>
       </c>
+      <c r="AB11">
+        <v>49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1250,6 +1289,9 @@
       <c r="AA12">
         <v>1</v>
       </c>
+      <c r="AB12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1355,6 +1397,9 @@
       <c r="AA13">
         <v>1</v>
       </c>
+      <c r="AB13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1442,6 +1487,9 @@
       <c r="AA14">
         <v>16</v>
       </c>
+      <c r="AB14">
+        <v>16</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1529,6 +1577,9 @@
       <c r="AA15">
         <v>29</v>
       </c>
+      <c r="AB15">
+        <v>29</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1648,6 +1699,11 @@
           <t/>
         </is>
       </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1749,6 +1805,11 @@
           <t/>
         </is>
       </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1872,6 +1933,9 @@
       <c r="AA18">
         <v>1</v>
       </c>
+      <c r="AB18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1965,6 +2029,9 @@
       <c r="AA19">
         <v>1</v>
       </c>
+      <c r="AB19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2050,6 +2117,9 @@
       <c r="AA20">
         <v>27</v>
       </c>
+      <c r="AB20">
+        <v>27</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2133,6 +2203,9 @@
         <v>86</v>
       </c>
       <c r="AA21">
+        <v>85</v>
+      </c>
+      <c r="AB21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-06 11:54 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -2118,7 +2118,7 @@
         <v>27</v>
       </c>
       <c r="AB20">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21">
@@ -2206,7 +2206,7 @@
         <v>85</v>
       </c>
       <c r="AB21">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-06 23:46 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -304,7 +304,7 @@
         <v>83</v>
       </c>
       <c r="AB2">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -568,7 +568,7 @@
         <v>37</v>
       </c>
       <c r="AB5">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -1186,7 +1186,7 @@
         <v>49</v>
       </c>
       <c r="AB11">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -1488,7 +1488,7 @@
         <v>16</v>
       </c>
       <c r="AB14">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -2206,7 +2206,7 @@
         <v>85</v>
       </c>
       <c r="AB21">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-07 01:56 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1186,7 +1186,7 @@
         <v>49</v>
       </c>
       <c r="AB11">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -1397,8 +1397,10 @@
       <c r="AA13">
         <v>1</v>
       </c>
-      <c r="AB13">
-        <v>1</v>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1488,7 +1490,7 @@
         <v>16</v>
       </c>
       <c r="AB14">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -1578,7 +1580,7 @@
         <v>29</v>
       </c>
       <c r="AB15">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -2029,8 +2031,10 @@
       <c r="AA19">
         <v>1</v>
       </c>
-      <c r="AB19">
-        <v>1</v>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2118,7 +2122,7 @@
         <v>27</v>
       </c>
       <c r="AB20">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-07 04:17 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -218,6 +218,11 @@
           <t>06/08/2026</t>
         </is>
       </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -306,6 +311,9 @@
       <c r="AB2">
         <v>84</v>
       </c>
+      <c r="AC2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -394,6 +402,9 @@
       <c r="AB3">
         <v>4</v>
       </c>
+      <c r="AC3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -482,6 +493,9 @@
       <c r="AB4">
         <v>2</v>
       </c>
+      <c r="AC4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -570,6 +584,9 @@
       <c r="AB5">
         <v>38</v>
       </c>
+      <c r="AC5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -658,6 +675,9 @@
       <c r="AB6">
         <v>31</v>
       </c>
+      <c r="AC6">
+        <v>31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -782,6 +802,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -888,6 +913,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1012,6 +1042,9 @@
       <c r="AB9">
         <v>2</v>
       </c>
+      <c r="AC9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1100,6 +1133,9 @@
       <c r="AB10">
         <v>7</v>
       </c>
+      <c r="AC10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1188,6 +1224,9 @@
       <c r="AB11">
         <v>46</v>
       </c>
+      <c r="AC11">
+        <v>46</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1292,6 +1331,9 @@
       <c r="AB12">
         <v>1</v>
       </c>
+      <c r="AC12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1402,6 +1444,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1492,6 +1539,9 @@
       <c r="AB14">
         <v>19</v>
       </c>
+      <c r="AC14">
+        <v>19</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1582,6 +1632,9 @@
       <c r="AB15">
         <v>25</v>
       </c>
+      <c r="AC15">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1706,6 +1759,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1812,6 +1870,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1938,6 +2001,9 @@
       <c r="AB18">
         <v>1</v>
       </c>
+      <c r="AC18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2036,6 +2102,11 @@
           <t/>
         </is>
       </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2124,6 +2195,9 @@
       <c r="AB20">
         <v>29</v>
       </c>
+      <c r="AC20">
+        <v>29</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2210,6 +2284,9 @@
         <v>85</v>
       </c>
       <c r="AB21">
+        <v>88</v>
+      </c>
+      <c r="AC21">
         <v>88</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-08 00:38 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1225,7 +1225,7 @@
         <v>46</v>
       </c>
       <c r="AC11">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -1444,10 +1444,8 @@
           <t/>
         </is>
       </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AC13">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1540,7 +1538,7 @@
         <v>19</v>
       </c>
       <c r="AC14">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
@@ -1633,7 +1631,7 @@
         <v>25</v>
       </c>
       <c r="AC15">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16">
@@ -2102,10 +2100,8 @@
           <t/>
         </is>
       </c>
-      <c r="AC19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AC19">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2196,7 +2192,7 @@
         <v>29</v>
       </c>
       <c r="AC20">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-08 03:14 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -223,6 +223,11 @@
           <t>07/08/2026</t>
         </is>
       </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -314,6 +319,9 @@
       <c r="AC2">
         <v>84</v>
       </c>
+      <c r="AD2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -405,6 +413,9 @@
       <c r="AC3">
         <v>4</v>
       </c>
+      <c r="AD3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -496,6 +507,9 @@
       <c r="AC4">
         <v>2</v>
       </c>
+      <c r="AD4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -587,6 +601,9 @@
       <c r="AC5">
         <v>38</v>
       </c>
+      <c r="AD5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -678,6 +695,9 @@
       <c r="AC6">
         <v>31</v>
       </c>
+      <c r="AD6">
+        <v>31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -807,6 +827,11 @@
           <t/>
         </is>
       </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -918,6 +943,11 @@
           <t/>
         </is>
       </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1045,6 +1075,9 @@
       <c r="AC9">
         <v>2</v>
       </c>
+      <c r="AD9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1136,6 +1169,9 @@
       <c r="AC10">
         <v>7</v>
       </c>
+      <c r="AD10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1227,6 +1263,9 @@
       <c r="AC11">
         <v>53</v>
       </c>
+      <c r="AD11">
+        <v>53</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1334,6 +1373,9 @@
       <c r="AC12">
         <v>1</v>
       </c>
+      <c r="AD12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1447,6 +1489,9 @@
       <c r="AC13">
         <v>1</v>
       </c>
+      <c r="AD13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1540,6 +1585,9 @@
       <c r="AC14">
         <v>18</v>
       </c>
+      <c r="AD14">
+        <v>18</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1633,6 +1681,9 @@
       <c r="AC15">
         <v>31</v>
       </c>
+      <c r="AD15">
+        <v>31</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1762,6 +1813,11 @@
           <t/>
         </is>
       </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1873,6 +1929,11 @@
           <t/>
         </is>
       </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2002,6 +2063,9 @@
       <c r="AC18">
         <v>1</v>
       </c>
+      <c r="AD18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2103,6 +2167,9 @@
       <c r="AC19">
         <v>1</v>
       </c>
+      <c r="AD19">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2194,6 +2261,9 @@
       <c r="AC20">
         <v>30</v>
       </c>
+      <c r="AD20">
+        <v>30</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2283,6 +2353,9 @@
         <v>88</v>
       </c>
       <c r="AC21">
+        <v>88</v>
+      </c>
+      <c r="AD21">
         <v>88</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-08 14:20 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1264,7 +1264,7 @@
         <v>53</v>
       </c>
       <c r="AD11">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -1586,7 +1586,7 @@
         <v>18</v>
       </c>
       <c r="AD14">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-09 00:41 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1264,7 +1264,7 @@
         <v>53</v>
       </c>
       <c r="AD11">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12">
@@ -1489,8 +1489,10 @@
       <c r="AC13">
         <v>1</v>
       </c>
-      <c r="AD13">
-        <v>1</v>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1586,7 +1588,7 @@
         <v>18</v>
       </c>
       <c r="AD14">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -1682,7 +1684,7 @@
         <v>31</v>
       </c>
       <c r="AD15">
-        <v>31</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -2168,7 +2170,7 @@
         <v>1</v>
       </c>
       <c r="AD19">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-09 03:22 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -228,6 +228,11 @@
           <t>08/08/2026</t>
         </is>
       </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>09/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -322,6 +327,9 @@
       <c r="AD2">
         <v>84</v>
       </c>
+      <c r="AE2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -416,6 +424,9 @@
       <c r="AD3">
         <v>4</v>
       </c>
+      <c r="AE3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -510,6 +521,9 @@
       <c r="AD4">
         <v>2</v>
       </c>
+      <c r="AE4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -604,6 +618,9 @@
       <c r="AD5">
         <v>38</v>
       </c>
+      <c r="AE5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -698,6 +715,9 @@
       <c r="AD6">
         <v>31</v>
       </c>
+      <c r="AE6">
+        <v>31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -832,6 +852,11 @@
           <t/>
         </is>
       </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -948,6 +973,11 @@
           <t/>
         </is>
       </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1078,6 +1108,9 @@
       <c r="AD9">
         <v>2</v>
       </c>
+      <c r="AE9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1172,6 +1205,9 @@
       <c r="AD10">
         <v>7</v>
       </c>
+      <c r="AE10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1266,6 +1302,9 @@
       <c r="AD11">
         <v>50</v>
       </c>
+      <c r="AE11">
+        <v>50</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1376,6 +1415,9 @@
       <c r="AD12">
         <v>1</v>
       </c>
+      <c r="AE12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1494,6 +1536,11 @@
           <t/>
         </is>
       </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1590,6 +1637,9 @@
       <c r="AD14">
         <v>19</v>
       </c>
+      <c r="AE14">
+        <v>19</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1686,6 +1736,9 @@
       <c r="AD15">
         <v>26</v>
       </c>
+      <c r="AE15">
+        <v>26</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1820,6 +1873,11 @@
           <t/>
         </is>
       </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1936,6 +1994,11 @@
           <t/>
         </is>
       </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2068,6 +2131,9 @@
       <c r="AD18">
         <v>1</v>
       </c>
+      <c r="AE18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2172,6 +2238,9 @@
       <c r="AD19">
         <v>3</v>
       </c>
+      <c r="AE19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2266,6 +2335,9 @@
       <c r="AD20">
         <v>30</v>
       </c>
+      <c r="AE20">
+        <v>30</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2358,6 +2430,9 @@
         <v>88</v>
       </c>
       <c r="AD21">
+        <v>88</v>
+      </c>
+      <c r="AE21">
         <v>88</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 00:42 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1303,7 +1303,7 @@
         <v>50</v>
       </c>
       <c r="AE11">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1415,8 +1415,10 @@
       <c r="AD12">
         <v>1</v>
       </c>
-      <c r="AE12">
-        <v>1</v>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1637,8 +1639,10 @@
       <c r="AD14">
         <v>19</v>
       </c>
-      <c r="AE14">
-        <v>19</v>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1737,7 +1741,7 @@
         <v>26</v>
       </c>
       <c r="AE15">
-        <v>26</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -2131,8 +2135,10 @@
       <c r="AD18">
         <v>1</v>
       </c>
-      <c r="AE18">
-        <v>1</v>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2238,8 +2244,10 @@
       <c r="AD19">
         <v>3</v>
       </c>
-      <c r="AE19">
-        <v>3</v>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2336,7 +2344,7 @@
         <v>30</v>
       </c>
       <c r="AE20">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">
@@ -2433,7 +2441,7 @@
         <v>88</v>
       </c>
       <c r="AE21">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 03:41 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -233,6 +233,11 @@
           <t>09/08/2026</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -330,6 +335,9 @@
       <c r="AE2">
         <v>84</v>
       </c>
+      <c r="AF2">
+        <v>84</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -427,6 +435,9 @@
       <c r="AE3">
         <v>4</v>
       </c>
+      <c r="AF3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -524,6 +535,9 @@
       <c r="AE4">
         <v>2</v>
       </c>
+      <c r="AF4">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -621,6 +635,9 @@
       <c r="AE5">
         <v>38</v>
       </c>
+      <c r="AF5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -718,6 +735,9 @@
       <c r="AE6">
         <v>31</v>
       </c>
+      <c r="AF6">
+        <v>31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -857,6 +877,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -978,6 +1003,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1111,6 +1141,9 @@
       <c r="AE9">
         <v>2</v>
       </c>
+      <c r="AF9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1208,6 +1241,9 @@
       <c r="AE10">
         <v>7</v>
       </c>
+      <c r="AF10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1305,6 +1341,9 @@
       <c r="AE11">
         <v>2</v>
       </c>
+      <c r="AF11">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1420,6 +1459,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1543,6 +1587,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1644,6 +1693,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1743,6 +1797,9 @@
       <c r="AE15">
         <v>2</v>
       </c>
+      <c r="AF15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1882,6 +1939,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2003,6 +2065,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2140,6 +2207,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2249,6 +2321,11 @@
           <t/>
         </is>
       </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2346,6 +2423,9 @@
       <c r="AE20">
         <v>29</v>
       </c>
+      <c r="AF20">
+        <v>29</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2441,6 +2521,9 @@
         <v>88</v>
       </c>
       <c r="AE21">
+        <v>86</v>
+      </c>
+      <c r="AF21">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 10:54 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1342,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="AF11">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1798,7 +1798,7 @@
         <v>2</v>
       </c>
       <c r="AF15">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 12:37 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1342,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="AF11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1797,8 +1797,10 @@
       <c r="AE15">
         <v>2</v>
       </c>
-      <c r="AF15">
-        <v>1</v>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 16:39 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -336,7 +336,7 @@
         <v>84</v>
       </c>
       <c r="AF2">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -736,7 +736,7 @@
         <v>31</v>
       </c>
       <c r="AF6">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -2526,7 +2526,7 @@
         <v>86</v>
       </c>
       <c r="AF21">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-10 22:23 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -336,7 +336,7 @@
         <v>84</v>
       </c>
       <c r="AF2">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         <v>2</v>
       </c>
       <c r="AF4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-11 00:42 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1342,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="AF11">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -1459,10 +1459,8 @@
           <t/>
         </is>
       </c>
-      <c r="AF12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF12">
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1587,10 +1585,8 @@
           <t/>
         </is>
       </c>
-      <c r="AF13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF13">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1693,10 +1689,8 @@
           <t/>
         </is>
       </c>
-      <c r="AF14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF14">
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -1797,10 +1791,8 @@
       <c r="AE15">
         <v>2</v>
       </c>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF15">
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -2209,10 +2201,8 @@
           <t/>
         </is>
       </c>
-      <c r="AF18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF18">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2323,10 +2313,8 @@
           <t/>
         </is>
       </c>
-      <c r="AF19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AF19">
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -2426,7 +2414,7 @@
         <v>29</v>
       </c>
       <c r="AF20">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-11 03:24 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -238,6 +238,11 @@
           <t>10/08/2026</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -338,6 +343,9 @@
       <c r="AF2">
         <v>82</v>
       </c>
+      <c r="AG2">
+        <v>82</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -438,6 +446,9 @@
       <c r="AF3">
         <v>4</v>
       </c>
+      <c r="AG3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -538,6 +549,9 @@
       <c r="AF4">
         <v>1</v>
       </c>
+      <c r="AG4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -638,6 +652,9 @@
       <c r="AF5">
         <v>38</v>
       </c>
+      <c r="AG5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -738,6 +755,9 @@
       <c r="AF6">
         <v>30</v>
       </c>
+      <c r="AG6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -882,6 +902,11 @@
           <t/>
         </is>
       </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1008,6 +1033,11 @@
           <t/>
         </is>
       </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1144,6 +1174,9 @@
       <c r="AF9">
         <v>2</v>
       </c>
+      <c r="AG9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1244,6 +1277,9 @@
       <c r="AF10">
         <v>7</v>
       </c>
+      <c r="AG10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1344,6 +1380,9 @@
       <c r="AF11">
         <v>49</v>
       </c>
+      <c r="AG11">
+        <v>49</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1462,6 +1501,9 @@
       <c r="AF12">
         <v>2</v>
       </c>
+      <c r="AG12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1588,6 +1630,9 @@
       <c r="AF13">
         <v>1</v>
       </c>
+      <c r="AG13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1692,6 +1737,9 @@
       <c r="AF14">
         <v>19</v>
       </c>
+      <c r="AG14">
+        <v>19</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1794,6 +1842,9 @@
       <c r="AF15">
         <v>23</v>
       </c>
+      <c r="AG15">
+        <v>23</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1938,6 +1989,11 @@
           <t/>
         </is>
       </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2064,6 +2120,11 @@
           <t/>
         </is>
       </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2204,6 +2265,9 @@
       <c r="AF18">
         <v>1</v>
       </c>
+      <c r="AG18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2316,6 +2380,9 @@
       <c r="AF19">
         <v>3</v>
       </c>
+      <c r="AG19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2416,6 +2483,9 @@
       <c r="AF20">
         <v>27</v>
       </c>
+      <c r="AG20">
+        <v>27</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2514,6 +2584,9 @@
         <v>86</v>
       </c>
       <c r="AF21">
+        <v>85</v>
+      </c>
+      <c r="AG21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-12 00:49 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1381,7 +1381,7 @@
         <v>49</v>
       </c>
       <c r="AG11">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -1738,7 +1738,7 @@
         <v>19</v>
       </c>
       <c r="AG14">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15">
@@ -1843,7 +1843,7 @@
         <v>23</v>
       </c>
       <c r="AG15">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
@@ -2484,7 +2484,7 @@
         <v>27</v>
       </c>
       <c r="AG20">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-12 03:52 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -243,6 +243,11 @@
           <t>11/08/2026</t>
         </is>
       </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -346,6 +351,9 @@
       <c r="AG2">
         <v>82</v>
       </c>
+      <c r="AH2">
+        <v>82</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -449,6 +457,9 @@
       <c r="AG3">
         <v>4</v>
       </c>
+      <c r="AH3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,6 +563,9 @@
       <c r="AG4">
         <v>1</v>
       </c>
+      <c r="AH4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -655,6 +669,9 @@
       <c r="AG5">
         <v>38</v>
       </c>
+      <c r="AH5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -758,6 +775,9 @@
       <c r="AG6">
         <v>30</v>
       </c>
+      <c r="AH6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -907,6 +927,11 @@
           <t/>
         </is>
       </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1038,6 +1063,11 @@
           <t/>
         </is>
       </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1177,6 +1207,9 @@
       <c r="AG9">
         <v>2</v>
       </c>
+      <c r="AH9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1280,6 +1313,9 @@
       <c r="AG10">
         <v>7</v>
       </c>
+      <c r="AH10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1383,6 +1419,9 @@
       <c r="AG11">
         <v>43</v>
       </c>
+      <c r="AH11">
+        <v>43</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1504,6 +1543,9 @@
       <c r="AG12">
         <v>2</v>
       </c>
+      <c r="AH12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1633,6 +1675,9 @@
       <c r="AG13">
         <v>1</v>
       </c>
+      <c r="AH13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1740,6 +1785,9 @@
       <c r="AG14">
         <v>17</v>
       </c>
+      <c r="AH14">
+        <v>17</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1845,6 +1893,9 @@
       <c r="AG15">
         <v>19</v>
       </c>
+      <c r="AH15">
+        <v>19</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1994,6 +2045,11 @@
           <t/>
         </is>
       </c>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2125,6 +2181,11 @@
           <t/>
         </is>
       </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2268,6 +2329,9 @@
       <c r="AG18">
         <v>1</v>
       </c>
+      <c r="AH18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2383,6 +2447,9 @@
       <c r="AG19">
         <v>3</v>
       </c>
+      <c r="AH19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2486,6 +2553,9 @@
       <c r="AG20">
         <v>21</v>
       </c>
+      <c r="AH20">
+        <v>21</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2587,6 +2657,9 @@
         <v>85</v>
       </c>
       <c r="AG21">
+        <v>85</v>
+      </c>
+      <c r="AH21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-12 12:37 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -352,7 +352,7 @@
         <v>82</v>
       </c>
       <c r="AH2">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -2660,7 +2660,7 @@
         <v>85</v>
       </c>
       <c r="AH21">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-12 14:48 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1420,7 +1420,7 @@
         <v>43</v>
       </c>
       <c r="AH11">
-        <v>43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1543,8 +1543,10 @@
       <c r="AG12">
         <v>2</v>
       </c>
-      <c r="AH12">
-        <v>2</v>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -1675,8 +1677,10 @@
       <c r="AG13">
         <v>1</v>
       </c>
-      <c r="AH13">
-        <v>1</v>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1785,8 +1789,10 @@
       <c r="AG14">
         <v>17</v>
       </c>
-      <c r="AH14">
-        <v>17</v>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -1893,8 +1899,10 @@
       <c r="AG15">
         <v>19</v>
       </c>
-      <c r="AH15">
-        <v>19</v>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -2329,8 +2337,10 @@
       <c r="AG18">
         <v>1</v>
       </c>
-      <c r="AH18">
-        <v>1</v>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2447,8 +2457,10 @@
       <c r="AG19">
         <v>3</v>
       </c>
-      <c r="AH19">
-        <v>3</v>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2554,7 +2566,7 @@
         <v>21</v>
       </c>
       <c r="AH20">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-13 03:56 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -248,6 +248,11 @@
           <t>12/08/2026</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -354,6 +359,9 @@
       <c r="AH2">
         <v>79</v>
       </c>
+      <c r="AI2">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -460,6 +468,9 @@
       <c r="AH3">
         <v>4</v>
       </c>
+      <c r="AI3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -566,6 +577,9 @@
       <c r="AH4">
         <v>1</v>
       </c>
+      <c r="AI4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -672,6 +686,9 @@
       <c r="AH5">
         <v>38</v>
       </c>
+      <c r="AI5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -778,6 +795,9 @@
       <c r="AH6">
         <v>30</v>
       </c>
+      <c r="AI6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -932,6 +952,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1068,6 +1093,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1210,6 +1240,9 @@
       <c r="AH9">
         <v>2</v>
       </c>
+      <c r="AI9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1316,6 +1349,9 @@
       <c r="AH10">
         <v>7</v>
       </c>
+      <c r="AI10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1422,6 +1458,9 @@
       <c r="AH11">
         <v>0</v>
       </c>
+      <c r="AI11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1548,6 +1587,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1682,6 +1726,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1794,6 +1843,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1904,6 +1958,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2058,6 +2117,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2194,6 +2258,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2342,6 +2411,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2462,6 +2536,11 @@
           <t/>
         </is>
       </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2568,6 +2647,9 @@
       <c r="AH20">
         <v>19</v>
       </c>
+      <c r="AI20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2672,6 +2754,9 @@
         <v>85</v>
       </c>
       <c r="AH21">
+        <v>86</v>
+      </c>
+      <c r="AI21">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-13 22:28 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -360,7 +360,7 @@
         <v>79</v>
       </c>
       <c r="AI2">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3">
@@ -1350,7 +1350,7 @@
         <v>7</v>
       </c>
       <c r="AI10">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -2757,7 +2757,7 @@
         <v>86</v>
       </c>
       <c r="AI21">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-14 03:52 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -253,6 +253,11 @@
           <t>13/08/2026</t>
         </is>
       </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>14/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -362,6 +367,9 @@
       <c r="AI2">
         <v>78</v>
       </c>
+      <c r="AJ2">
+        <v>78</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -471,6 +479,9 @@
       <c r="AI3">
         <v>4</v>
       </c>
+      <c r="AJ3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -580,6 +591,9 @@
       <c r="AI4">
         <v>1</v>
       </c>
+      <c r="AJ4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -689,6 +703,9 @@
       <c r="AI5">
         <v>38</v>
       </c>
+      <c r="AJ5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -798,6 +815,9 @@
       <c r="AI6">
         <v>30</v>
       </c>
+      <c r="AJ6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -957,6 +977,11 @@
           <t/>
         </is>
       </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1098,6 +1123,11 @@
           <t/>
         </is>
       </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1243,6 +1273,9 @@
       <c r="AI9">
         <v>2</v>
       </c>
+      <c r="AJ9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1352,6 +1385,9 @@
       <c r="AI10">
         <v>6</v>
       </c>
+      <c r="AJ10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1461,6 +1497,9 @@
       <c r="AI11">
         <v>0</v>
       </c>
+      <c r="AJ11">
+        <v>58</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1592,6 +1631,9 @@
           <t/>
         </is>
       </c>
+      <c r="AJ12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1731,6 +1773,11 @@
           <t/>
         </is>
       </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1848,6 +1895,9 @@
           <t/>
         </is>
       </c>
+      <c r="AJ14">
+        <v>29</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1963,6 +2013,9 @@
           <t/>
         </is>
       </c>
+      <c r="AJ15">
+        <v>24</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2122,6 +2175,11 @@
           <t/>
         </is>
       </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2263,6 +2321,11 @@
           <t/>
         </is>
       </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2416,6 +2479,9 @@
           <t/>
         </is>
       </c>
+      <c r="AJ18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2541,6 +2607,9 @@
           <t/>
         </is>
       </c>
+      <c r="AJ19">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2650,6 +2719,9 @@
       <c r="AI20">
         <v>10</v>
       </c>
+      <c r="AJ20">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2757,6 +2829,9 @@
         <v>86</v>
       </c>
       <c r="AI21">
+        <v>85</v>
+      </c>
+      <c r="AJ21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-15 00:28 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="AJ14">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -2014,7 +2014,7 @@
         </is>
       </c>
       <c r="AJ15">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-15 04:17 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -258,6 +258,11 @@
           <t>14/08/2026</t>
         </is>
       </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>15/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -370,6 +375,9 @@
       <c r="AJ2">
         <v>79</v>
       </c>
+      <c r="AK2">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -482,6 +490,9 @@
       <c r="AJ3">
         <v>4</v>
       </c>
+      <c r="AK3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -594,6 +605,9 @@
       <c r="AJ4">
         <v>1</v>
       </c>
+      <c r="AK4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -706,6 +720,9 @@
       <c r="AJ5">
         <v>38</v>
       </c>
+      <c r="AK5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -818,6 +835,9 @@
       <c r="AJ6">
         <v>30</v>
       </c>
+      <c r="AK6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -982,6 +1002,11 @@
           <t/>
         </is>
       </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1128,6 +1153,11 @@
           <t/>
         </is>
       </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1276,6 +1306,9 @@
       <c r="AJ9">
         <v>2</v>
       </c>
+      <c r="AK9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1388,6 +1421,9 @@
       <c r="AJ10">
         <v>6</v>
       </c>
+      <c r="AK10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1500,6 +1536,9 @@
       <c r="AJ11">
         <v>58</v>
       </c>
+      <c r="AK11">
+        <v>58</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1634,6 +1673,9 @@
       <c r="AJ12">
         <v>2</v>
       </c>
+      <c r="AK12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1778,6 +1820,11 @@
           <t/>
         </is>
       </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1898,6 +1945,9 @@
       <c r="AJ14">
         <v>28</v>
       </c>
+      <c r="AK14">
+        <v>28</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2016,6 +2066,9 @@
       <c r="AJ15">
         <v>25</v>
       </c>
+      <c r="AK15">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2180,6 +2233,11 @@
           <t/>
         </is>
       </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2326,6 +2384,11 @@
           <t/>
         </is>
       </c>
+      <c r="AK17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2482,6 +2545,9 @@
       <c r="AJ18">
         <v>1</v>
       </c>
+      <c r="AK18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2610,6 +2676,9 @@
       <c r="AJ19">
         <v>2</v>
       </c>
+      <c r="AK19">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2722,6 +2791,9 @@
       <c r="AJ20">
         <v>18</v>
       </c>
+      <c r="AK20">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2832,6 +2904,9 @@
         <v>85</v>
       </c>
       <c r="AJ21">
+        <v>85</v>
+      </c>
+      <c r="AK21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-16 00:29 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1537,7 +1537,7 @@
         <v>58</v>
       </c>
       <c r="AK11">
-        <v>58</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
@@ -1946,7 +1946,7 @@
         <v>28</v>
       </c>
       <c r="AK14">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -2067,7 +2067,7 @@
         <v>25</v>
       </c>
       <c r="AK15">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
@@ -2545,8 +2545,10 @@
       <c r="AJ18">
         <v>1</v>
       </c>
-      <c r="AK18">
-        <v>1</v>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -2792,7 +2794,7 @@
         <v>18</v>
       </c>
       <c r="AK20">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-16 04:23 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -263,6 +263,11 @@
           <t>15/08/2026</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>16/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -378,6 +383,9 @@
       <c r="AK2">
         <v>79</v>
       </c>
+      <c r="AL2">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +501,9 @@
       <c r="AK3">
         <v>4</v>
       </c>
+      <c r="AL3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -608,6 +619,9 @@
       <c r="AK4">
         <v>1</v>
       </c>
+      <c r="AL4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -723,6 +737,9 @@
       <c r="AK5">
         <v>38</v>
       </c>
+      <c r="AL5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -838,6 +855,9 @@
       <c r="AK6">
         <v>30</v>
       </c>
+      <c r="AL6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1007,6 +1027,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1158,6 +1183,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1309,6 +1339,9 @@
       <c r="AK9">
         <v>2</v>
       </c>
+      <c r="AL9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1424,6 +1457,9 @@
       <c r="AK10">
         <v>6</v>
       </c>
+      <c r="AL10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1539,6 +1575,9 @@
       <c r="AK11">
         <v>43</v>
       </c>
+      <c r="AL11">
+        <v>43</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1676,6 +1715,9 @@
       <c r="AK12">
         <v>2</v>
       </c>
+      <c r="AL12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1825,6 +1867,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1948,6 +1995,9 @@
       <c r="AK14">
         <v>20</v>
       </c>
+      <c r="AL14">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2069,6 +2119,9 @@
       <c r="AK15">
         <v>19</v>
       </c>
+      <c r="AL15">
+        <v>19</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2238,6 +2291,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2389,6 +2447,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2550,6 +2613,11 @@
           <t/>
         </is>
       </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2681,6 +2749,9 @@
       <c r="AK19">
         <v>2</v>
       </c>
+      <c r="AL19">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2796,6 +2867,9 @@
       <c r="AK20">
         <v>19</v>
       </c>
+      <c r="AL20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2909,6 +2983,9 @@
         <v>85</v>
       </c>
       <c r="AK21">
+        <v>85</v>
+      </c>
+      <c r="AL21">
         <v>85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 00:27 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1576,7 +1576,7 @@
         <v>43</v>
       </c>
       <c r="AL11">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -1716,7 +1716,7 @@
         <v>2</v>
       </c>
       <c r="AL12">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -1996,7 +1996,7 @@
         <v>20</v>
       </c>
       <c r="AL14">
-        <v>20</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15">
@@ -2120,7 +2120,7 @@
         <v>19</v>
       </c>
       <c r="AL15">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -2613,10 +2613,8 @@
           <t/>
         </is>
       </c>
-      <c r="AL18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AL18">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2986,7 +2984,7 @@
         <v>85</v>
       </c>
       <c r="AL21">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 04:29 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -268,6 +268,11 @@
           <t>16/08/2026</t>
         </is>
       </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -386,6 +391,9 @@
       <c r="AL2">
         <v>79</v>
       </c>
+      <c r="AM2">
+        <v>79</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -504,6 +512,9 @@
       <c r="AL3">
         <v>4</v>
       </c>
+      <c r="AM3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -622,6 +633,9 @@
       <c r="AL4">
         <v>1</v>
       </c>
+      <c r="AM4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -740,6 +754,9 @@
       <c r="AL5">
         <v>38</v>
       </c>
+      <c r="AM5">
+        <v>38</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -858,6 +875,9 @@
       <c r="AL6">
         <v>30</v>
       </c>
+      <c r="AM6">
+        <v>30</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1032,6 +1052,11 @@
           <t/>
         </is>
       </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1188,6 +1213,11 @@
           <t/>
         </is>
       </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1342,6 +1372,9 @@
       <c r="AL9">
         <v>2</v>
       </c>
+      <c r="AM9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1460,6 +1493,9 @@
       <c r="AL10">
         <v>6</v>
       </c>
+      <c r="AM10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1578,6 +1614,9 @@
       <c r="AL11">
         <v>51</v>
       </c>
+      <c r="AM11">
+        <v>51</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1718,6 +1757,9 @@
       <c r="AL12">
         <v>4</v>
       </c>
+      <c r="AM12">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1872,6 +1914,11 @@
           <t/>
         </is>
       </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1998,6 +2045,9 @@
       <c r="AL14">
         <v>26</v>
       </c>
+      <c r="AM14">
+        <v>26</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2122,6 +2172,9 @@
       <c r="AL15">
         <v>18</v>
       </c>
+      <c r="AM15">
+        <v>18</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2296,6 +2349,11 @@
           <t/>
         </is>
       </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2452,6 +2510,11 @@
           <t/>
         </is>
       </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2616,6 +2679,9 @@
       <c r="AL18">
         <v>1</v>
       </c>
+      <c r="AM18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2750,6 +2816,9 @@
       <c r="AL19">
         <v>2</v>
       </c>
+      <c r="AM19">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2868,6 +2937,9 @@
       <c r="AL20">
         <v>19</v>
       </c>
+      <c r="AM20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2984,6 +3056,9 @@
         <v>85</v>
       </c>
       <c r="AL21">
+        <v>83</v>
+      </c>
+      <c r="AM21">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 14:15 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -392,7 +392,7 @@
         <v>79</v>
       </c>
       <c r="AM2">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
@@ -1494,7 +1494,7 @@
         <v>6</v>
       </c>
       <c r="AM10">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -1615,7 +1615,7 @@
         <v>51</v>
       </c>
       <c r="AM11">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12">
@@ -2817,7 +2817,7 @@
         <v>2</v>
       </c>
       <c r="AM19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -3059,7 +3059,7 @@
         <v>83</v>
       </c>
       <c r="AM21">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 16:12 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1615,7 +1615,7 @@
         <v>51</v>
       </c>
       <c r="AM11">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
@@ -2817,7 +2817,7 @@
         <v>2</v>
       </c>
       <c r="AM19">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -3059,7 +3059,7 @@
         <v>83</v>
       </c>
       <c r="AM21">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 20:11 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -392,7 +392,7 @@
         <v>79</v>
       </c>
       <c r="AM2">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -755,7 +755,7 @@
         <v>38</v>
       </c>
       <c r="AM5">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -876,7 +876,7 @@
         <v>30</v>
       </c>
       <c r="AM6">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -1615,7 +1615,7 @@
         <v>51</v>
       </c>
       <c r="AM11">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12">
@@ -2173,7 +2173,7 @@
         <v>18</v>
       </c>
       <c r="AM15">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16">
@@ -2938,7 +2938,7 @@
         <v>19</v>
       </c>
       <c r="AM20">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -3059,7 +3059,7 @@
         <v>83</v>
       </c>
       <c r="AM21">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-17 22:10 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -392,7 +392,7 @@
         <v>79</v>
       </c>
       <c r="AM2">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -513,7 +513,7 @@
         <v>4</v>
       </c>
       <c r="AM3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -755,7 +755,7 @@
         <v>38</v>
       </c>
       <c r="AM5">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -1373,7 +1373,7 @@
         <v>2</v>
       </c>
       <c r="AM9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -1615,7 +1615,7 @@
         <v>51</v>
       </c>
       <c r="AM11">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -1758,7 +1758,7 @@
         <v>4</v>
       </c>
       <c r="AM12">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -2046,7 +2046,7 @@
         <v>26</v>
       </c>
       <c r="AM14">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -2173,7 +2173,7 @@
         <v>18</v>
       </c>
       <c r="AM15">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
@@ -3059,7 +3059,7 @@
         <v>83</v>
       </c>
       <c r="AM21">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-18 00:26 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -392,7 +392,7 @@
         <v>79</v>
       </c>
       <c r="AM2">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -755,7 +755,7 @@
         <v>38</v>
       </c>
       <c r="AM5">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -876,7 +876,7 @@
         <v>30</v>
       </c>
       <c r="AM6">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -1615,7 +1615,7 @@
         <v>51</v>
       </c>
       <c r="AM11">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12">
@@ -1758,7 +1758,7 @@
         <v>4</v>
       </c>
       <c r="AM12">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -2173,7 +2173,7 @@
         <v>18</v>
       </c>
       <c r="AM15">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -2817,7 +2817,7 @@
         <v>2</v>
       </c>
       <c r="AM19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -2938,7 +2938,7 @@
         <v>19</v>
       </c>
       <c r="AM20">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-18 04:26 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -273,6 +273,11 @@
           <t>17/08/2026</t>
         </is>
       </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -394,6 +399,9 @@
       <c r="AM2">
         <v>85</v>
       </c>
+      <c r="AN2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,6 +523,9 @@
       <c r="AM3">
         <v>3</v>
       </c>
+      <c r="AN3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -636,6 +647,9 @@
       <c r="AM4">
         <v>1</v>
       </c>
+      <c r="AN4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -757,6 +771,9 @@
       <c r="AM5">
         <v>39</v>
       </c>
+      <c r="AN5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -878,6 +895,9 @@
       <c r="AM6">
         <v>32</v>
       </c>
+      <c r="AN6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1057,6 +1077,11 @@
           <t/>
         </is>
       </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1218,6 +1243,11 @@
           <t/>
         </is>
       </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1375,6 +1405,9 @@
       <c r="AM9">
         <v>3</v>
       </c>
+      <c r="AN9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1496,6 +1529,9 @@
       <c r="AM10">
         <v>7</v>
       </c>
+      <c r="AN10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1617,6 +1653,9 @@
       <c r="AM11">
         <v>57</v>
       </c>
+      <c r="AN11">
+        <v>57</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1760,6 +1799,9 @@
       <c r="AM12">
         <v>2</v>
       </c>
+      <c r="AN12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1919,6 +1961,11 @@
           <t/>
         </is>
       </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2048,6 +2095,9 @@
       <c r="AM14">
         <v>27</v>
       </c>
+      <c r="AN14">
+        <v>27</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2175,6 +2225,9 @@
       <c r="AM15">
         <v>24</v>
       </c>
+      <c r="AN15">
+        <v>24</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2354,6 +2407,11 @@
           <t/>
         </is>
       </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2515,6 +2573,11 @@
           <t/>
         </is>
       </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2682,6 +2745,9 @@
       <c r="AM18">
         <v>1</v>
       </c>
+      <c r="AN18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2819,6 +2885,9 @@
       <c r="AM19">
         <v>3</v>
       </c>
+      <c r="AN19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2940,6 +3009,9 @@
       <c r="AM20">
         <v>20</v>
       </c>
+      <c r="AN20">
+        <v>20</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3059,6 +3131,9 @@
         <v>83</v>
       </c>
       <c r="AM21">
+        <v>90</v>
+      </c>
+      <c r="AN21">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-19 00:26 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1654,7 +1654,7 @@
         <v>57</v>
       </c>
       <c r="AN11">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12">
@@ -1800,7 +1800,7 @@
         <v>2</v>
       </c>
       <c r="AN12">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -2096,7 +2096,7 @@
         <v>27</v>
       </c>
       <c r="AN14">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
@@ -2226,7 +2226,7 @@
         <v>24</v>
       </c>
       <c r="AN15">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -3010,7 +3010,7 @@
         <v>20</v>
       </c>
       <c r="AN20">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-19 04:24 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -278,6 +278,11 @@
           <t>18/08/2026</t>
         </is>
       </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>19/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -402,6 +407,9 @@
       <c r="AN2">
         <v>85</v>
       </c>
+      <c r="AO2">
+        <v>85</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -526,6 +534,9 @@
       <c r="AN3">
         <v>3</v>
       </c>
+      <c r="AO3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -650,6 +661,9 @@
       <c r="AN4">
         <v>1</v>
       </c>
+      <c r="AO4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -774,6 +788,9 @@
       <c r="AN5">
         <v>39</v>
       </c>
+      <c r="AO5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -898,6 +915,9 @@
       <c r="AN6">
         <v>32</v>
       </c>
+      <c r="AO6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1082,6 +1102,11 @@
           <t/>
         </is>
       </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1248,6 +1273,11 @@
           <t/>
         </is>
       </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1408,6 +1438,9 @@
       <c r="AN9">
         <v>3</v>
       </c>
+      <c r="AO9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1532,6 +1565,9 @@
       <c r="AN10">
         <v>7</v>
       </c>
+      <c r="AO10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1656,6 +1692,9 @@
       <c r="AN11">
         <v>64</v>
       </c>
+      <c r="AO11">
+        <v>64</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1802,6 +1841,9 @@
       <c r="AN12">
         <v>3</v>
       </c>
+      <c r="AO12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1966,6 +2008,11 @@
           <t/>
         </is>
       </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2098,6 +2145,9 @@
       <c r="AN14">
         <v>32</v>
       </c>
+      <c r="AO14">
+        <v>32</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2228,6 +2278,9 @@
       <c r="AN15">
         <v>25</v>
       </c>
+      <c r="AO15">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2412,6 +2465,11 @@
           <t/>
         </is>
       </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2578,6 +2636,11 @@
           <t/>
         </is>
       </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2748,6 +2811,9 @@
       <c r="AN18">
         <v>1</v>
       </c>
+      <c r="AO18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2888,6 +2954,9 @@
       <c r="AN19">
         <v>3</v>
       </c>
+      <c r="AO19">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3012,6 +3081,9 @@
       <c r="AN20">
         <v>20</v>
       </c>
+      <c r="AO20">
+        <v>20</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3134,6 +3206,9 @@
         <v>90</v>
       </c>
       <c r="AN21">
+        <v>90</v>
+      </c>
+      <c r="AO21">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-19 16:15 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -408,7 +408,7 @@
         <v>85</v>
       </c>
       <c r="AO2">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -1439,7 +1439,7 @@
         <v>3</v>
       </c>
       <c r="AO9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -3209,7 +3209,7 @@
         <v>90</v>
       </c>
       <c r="AO21">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-20 00:27 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1693,7 +1693,7 @@
         <v>64</v>
       </c>
       <c r="AO11">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12">
@@ -2279,7 +2279,7 @@
         <v>25</v>
       </c>
       <c r="AO15">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -2812,7 +2812,7 @@
         <v>1</v>
       </c>
       <c r="AO18">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -2955,7 +2955,7 @@
         <v>3</v>
       </c>
       <c r="AO19">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -3082,7 +3082,7 @@
         <v>20</v>
       </c>
       <c r="AO20">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-20 04:23 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -283,6 +283,11 @@
           <t>19/08/2026</t>
         </is>
       </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>20/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -410,6 +415,9 @@
       <c r="AO2">
         <v>86</v>
       </c>
+      <c r="AP2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,6 +545,9 @@
       <c r="AO3">
         <v>3</v>
       </c>
+      <c r="AP3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -664,6 +675,9 @@
       <c r="AO4">
         <v>1</v>
       </c>
+      <c r="AP4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -791,6 +805,9 @@
       <c r="AO5">
         <v>39</v>
       </c>
+      <c r="AP5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -918,6 +935,9 @@
       <c r="AO6">
         <v>32</v>
       </c>
+      <c r="AP6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1107,6 +1127,11 @@
           <t/>
         </is>
       </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1278,6 +1303,11 @@
           <t/>
         </is>
       </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1441,6 +1471,9 @@
       <c r="AO9">
         <v>4</v>
       </c>
+      <c r="AP9">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1568,6 +1601,9 @@
       <c r="AO10">
         <v>7</v>
       </c>
+      <c r="AP10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1695,6 +1731,9 @@
       <c r="AO11">
         <v>65</v>
       </c>
+      <c r="AP11">
+        <v>65</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1844,6 +1883,9 @@
       <c r="AO12">
         <v>3</v>
       </c>
+      <c r="AP12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2013,6 +2055,11 @@
           <t/>
         </is>
       </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2148,6 +2195,9 @@
       <c r="AO14">
         <v>32</v>
       </c>
+      <c r="AP14">
+        <v>32</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2281,6 +2331,9 @@
       <c r="AO15">
         <v>24</v>
       </c>
+      <c r="AP15">
+        <v>24</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2470,6 +2523,11 @@
           <t/>
         </is>
       </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2641,6 +2699,11 @@
           <t/>
         </is>
       </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2814,6 +2877,9 @@
       <c r="AO18">
         <v>2</v>
       </c>
+      <c r="AP18">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2957,6 +3023,9 @@
       <c r="AO19">
         <v>4</v>
       </c>
+      <c r="AP19">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3084,6 +3153,9 @@
       <c r="AO20">
         <v>21</v>
       </c>
+      <c r="AP20">
+        <v>21</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3209,6 +3281,9 @@
         <v>90</v>
       </c>
       <c r="AO21">
+        <v>91</v>
+      </c>
+      <c r="AP21">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-21 00:30 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -2332,7 +2332,7 @@
         <v>24</v>
       </c>
       <c r="AP15">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
@@ -2878,7 +2878,7 @@
         <v>2</v>
       </c>
       <c r="AP18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -3154,7 +3154,7 @@
         <v>21</v>
       </c>
       <c r="AP20">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-21 04:25 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -288,6 +288,11 @@
           <t>20/08/2026</t>
         </is>
       </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>21/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -418,6 +423,9 @@
       <c r="AP2">
         <v>86</v>
       </c>
+      <c r="AQ2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -548,6 +556,9 @@
       <c r="AP3">
         <v>3</v>
       </c>
+      <c r="AQ3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -678,6 +689,9 @@
       <c r="AP4">
         <v>1</v>
       </c>
+      <c r="AQ4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -808,6 +822,9 @@
       <c r="AP5">
         <v>39</v>
       </c>
+      <c r="AQ5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -938,6 +955,9 @@
       <c r="AP6">
         <v>32</v>
       </c>
+      <c r="AQ6">
+        <v>32</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1132,6 +1152,11 @@
           <t/>
         </is>
       </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1308,6 +1333,11 @@
           <t/>
         </is>
       </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1474,6 +1504,9 @@
       <c r="AP9">
         <v>4</v>
       </c>
+      <c r="AQ9">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1604,6 +1637,9 @@
       <c r="AP10">
         <v>7</v>
       </c>
+      <c r="AQ10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1734,6 +1770,9 @@
       <c r="AP11">
         <v>65</v>
       </c>
+      <c r="AQ11">
+        <v>65</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1886,6 +1925,9 @@
       <c r="AP12">
         <v>3</v>
       </c>
+      <c r="AQ12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2060,6 +2102,11 @@
           <t/>
         </is>
       </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2198,6 +2245,9 @@
       <c r="AP14">
         <v>32</v>
       </c>
+      <c r="AQ14">
+        <v>32</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2334,6 +2384,9 @@
       <c r="AP15">
         <v>25</v>
       </c>
+      <c r="AQ15">
+        <v>25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2528,6 +2581,11 @@
           <t/>
         </is>
       </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2704,6 +2762,11 @@
           <t/>
         </is>
       </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2880,6 +2943,9 @@
       <c r="AP18">
         <v>1</v>
       </c>
+      <c r="AQ18">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3026,6 +3092,9 @@
       <c r="AP19">
         <v>4</v>
       </c>
+      <c r="AQ19">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3156,6 +3225,9 @@
       <c r="AP20">
         <v>19</v>
       </c>
+      <c r="AQ20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3284,6 +3356,9 @@
         <v>91</v>
       </c>
       <c r="AP21">
+        <v>91</v>
+      </c>
+      <c r="AQ21">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-21 16:17 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -424,7 +424,7 @@
         <v>86</v>
       </c>
       <c r="AQ2">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3">
@@ -956,7 +956,7 @@
         <v>32</v>
       </c>
       <c r="AQ6">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -1771,7 +1771,7 @@
         <v>65</v>
       </c>
       <c r="AQ11">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
@@ -2385,7 +2385,7 @@
         <v>25</v>
       </c>
       <c r="AQ15">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -3359,7 +3359,7 @@
         <v>91</v>
       </c>
       <c r="AQ21">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-21 20:10 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -424,7 +424,7 @@
         <v>86</v>
       </c>
       <c r="AQ2">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -1505,7 +1505,7 @@
         <v>4</v>
       </c>
       <c r="AQ9">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -3359,7 +3359,7 @@
         <v>91</v>
       </c>
       <c r="AQ21">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-22 00:27 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1771,7 +1771,7 @@
         <v>65</v>
       </c>
       <c r="AQ11">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -2102,10 +2102,8 @@
           <t/>
         </is>
       </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AQ13">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -2246,7 +2244,7 @@
         <v>32</v>
       </c>
       <c r="AQ14">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -2385,7 +2383,7 @@
         <v>25</v>
       </c>
       <c r="AQ15">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -2944,7 +2942,7 @@
         <v>1</v>
       </c>
       <c r="AQ18">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -3226,7 +3224,7 @@
         <v>19</v>
       </c>
       <c r="AQ20">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-22 04:19 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -293,6 +293,11 @@
           <t>21/08/2026</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -426,6 +431,9 @@
       <c r="AQ2">
         <v>86</v>
       </c>
+      <c r="AR2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -559,6 +567,9 @@
       <c r="AQ3">
         <v>3</v>
       </c>
+      <c r="AR3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -692,6 +703,9 @@
       <c r="AQ4">
         <v>1</v>
       </c>
+      <c r="AR4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -825,6 +839,9 @@
       <c r="AQ5">
         <v>39</v>
       </c>
+      <c r="AR5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -958,6 +975,9 @@
       <c r="AQ6">
         <v>33</v>
       </c>
+      <c r="AR6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1157,6 +1177,11 @@
           <t/>
         </is>
       </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1338,6 +1363,11 @@
           <t/>
         </is>
       </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1507,6 +1537,9 @@
       <c r="AQ9">
         <v>3</v>
       </c>
+      <c r="AR9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1640,6 +1673,9 @@
       <c r="AQ10">
         <v>7</v>
       </c>
+      <c r="AR10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1773,6 +1809,9 @@
       <c r="AQ11">
         <v>63</v>
       </c>
+      <c r="AR11">
+        <v>63</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1928,6 +1967,9 @@
       <c r="AQ12">
         <v>3</v>
       </c>
+      <c r="AR12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2105,6 +2147,9 @@
       <c r="AQ13">
         <v>1</v>
       </c>
+      <c r="AR13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2246,6 +2291,9 @@
       <c r="AQ14">
         <v>29</v>
       </c>
+      <c r="AR14">
+        <v>29</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2385,6 +2433,9 @@
       <c r="AQ15">
         <v>23</v>
       </c>
+      <c r="AR15">
+        <v>23</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2584,6 +2635,11 @@
           <t/>
         </is>
       </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2765,6 +2821,11 @@
           <t/>
         </is>
       </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2944,6 +3005,9 @@
       <c r="AQ18">
         <v>3</v>
       </c>
+      <c r="AR18">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3093,6 +3157,9 @@
       <c r="AQ19">
         <v>4</v>
       </c>
+      <c r="AR19">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3226,6 +3293,9 @@
       <c r="AQ20">
         <v>18</v>
       </c>
+      <c r="AR20">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3357,6 +3427,9 @@
         <v>91</v>
       </c>
       <c r="AQ21">
+        <v>91</v>
+      </c>
+      <c r="AR21">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-22 14:09 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1810,7 +1810,7 @@
         <v>63</v>
       </c>
       <c r="AR11">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
@@ -2292,7 +2292,7 @@
         <v>29</v>
       </c>
       <c r="AR14">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-23 00:30 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1810,7 +1810,7 @@
         <v>63</v>
       </c>
       <c r="AR11">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12">
@@ -2292,7 +2292,7 @@
         <v>29</v>
       </c>
       <c r="AR14">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -3158,7 +3158,7 @@
         <v>4</v>
       </c>
       <c r="AR19">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-23 04:25 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -298,6 +298,11 @@
           <t>22/08/2026</t>
         </is>
       </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>23/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -434,6 +439,9 @@
       <c r="AR2">
         <v>86</v>
       </c>
+      <c r="AS2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -570,6 +578,9 @@
       <c r="AR3">
         <v>3</v>
       </c>
+      <c r="AS3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -706,6 +717,9 @@
       <c r="AR4">
         <v>1</v>
       </c>
+      <c r="AS4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -842,6 +856,9 @@
       <c r="AR5">
         <v>39</v>
       </c>
+      <c r="AS5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -978,6 +995,9 @@
       <c r="AR6">
         <v>33</v>
       </c>
+      <c r="AS6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1182,6 +1202,11 @@
           <t/>
         </is>
       </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1368,6 +1393,11 @@
           <t/>
         </is>
       </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1540,6 +1570,9 @@
       <c r="AR9">
         <v>3</v>
       </c>
+      <c r="AS9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1676,6 +1709,9 @@
       <c r="AR10">
         <v>7</v>
       </c>
+      <c r="AS10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1812,6 +1848,9 @@
       <c r="AR11">
         <v>66</v>
       </c>
+      <c r="AS11">
+        <v>66</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1970,6 +2009,9 @@
       <c r="AR12">
         <v>3</v>
       </c>
+      <c r="AS12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2150,6 +2192,9 @@
       <c r="AR13">
         <v>1</v>
       </c>
+      <c r="AS13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2294,6 +2339,9 @@
       <c r="AR14">
         <v>31</v>
       </c>
+      <c r="AS14">
+        <v>31</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2436,6 +2484,9 @@
       <c r="AR15">
         <v>23</v>
       </c>
+      <c r="AS15">
+        <v>23</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2640,6 +2691,11 @@
           <t/>
         </is>
       </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2826,6 +2882,11 @@
           <t/>
         </is>
       </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3008,6 +3069,9 @@
       <c r="AR18">
         <v>3</v>
       </c>
+      <c r="AS18">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3160,6 +3224,9 @@
       <c r="AR19">
         <v>5</v>
       </c>
+      <c r="AS19">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3296,6 +3363,9 @@
       <c r="AR20">
         <v>18</v>
       </c>
+      <c r="AS20">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3430,6 +3500,9 @@
         <v>91</v>
       </c>
       <c r="AR21">
+        <v>91</v>
+      </c>
+      <c r="AS21">
         <v>91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-24 00:28 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1849,7 +1849,7 @@
         <v>66</v>
       </c>
       <c r="AS11">
-        <v>66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2009,8 +2009,10 @@
       <c r="AR12">
         <v>3</v>
       </c>
-      <c r="AS12">
-        <v>3</v>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2192,8 +2194,10 @@
       <c r="AR13">
         <v>1</v>
       </c>
-      <c r="AS13">
-        <v>1</v>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -2339,8 +2343,10 @@
       <c r="AR14">
         <v>31</v>
       </c>
-      <c r="AS14">
-        <v>31</v>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2484,8 +2490,10 @@
       <c r="AR15">
         <v>23</v>
       </c>
-      <c r="AS15">
-        <v>23</v>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -3069,8 +3077,10 @@
       <c r="AR18">
         <v>3</v>
       </c>
-      <c r="AS18">
-        <v>3</v>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -3224,8 +3234,10 @@
       <c r="AR19">
         <v>5</v>
       </c>
-      <c r="AS19">
-        <v>5</v>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -3364,7 +3376,7 @@
         <v>18</v>
       </c>
       <c r="AS20">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21">
@@ -3503,7 +3515,7 @@
         <v>91</v>
       </c>
       <c r="AS21">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-24 04:32 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -303,6 +303,11 @@
           <t>23/08/2026</t>
         </is>
       </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -442,6 +447,9 @@
       <c r="AS2">
         <v>86</v>
       </c>
+      <c r="AT2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -581,6 +589,9 @@
       <c r="AS3">
         <v>3</v>
       </c>
+      <c r="AT3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -720,6 +731,9 @@
       <c r="AS4">
         <v>1</v>
       </c>
+      <c r="AT4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -859,6 +873,9 @@
       <c r="AS5">
         <v>39</v>
       </c>
+      <c r="AT5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -998,6 +1015,9 @@
       <c r="AS6">
         <v>33</v>
       </c>
+      <c r="AT6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1207,6 +1227,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1398,6 +1423,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1573,6 +1603,9 @@
       <c r="AS9">
         <v>3</v>
       </c>
+      <c r="AT9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1712,6 +1745,9 @@
       <c r="AS10">
         <v>7</v>
       </c>
+      <c r="AT10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1851,6 +1887,9 @@
       <c r="AS11">
         <v>0</v>
       </c>
+      <c r="AT11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2014,6 +2053,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2199,6 +2243,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2348,6 +2397,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2495,6 +2549,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2704,6 +2763,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2895,6 +2959,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3082,6 +3151,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3239,6 +3313,11 @@
           <t/>
         </is>
       </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3378,6 +3457,9 @@
       <c r="AS20">
         <v>16</v>
       </c>
+      <c r="AT20">
+        <v>16</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3515,6 +3597,9 @@
         <v>91</v>
       </c>
       <c r="AS21">
+        <v>90</v>
+      </c>
+      <c r="AT21">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-08-25 00:28 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="AT11">
-        <v>0</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12">
@@ -2053,10 +2053,8 @@
           <t/>
         </is>
       </c>
-      <c r="AT12" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AT12">
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -2397,10 +2395,8 @@
           <t/>
         </is>
       </c>
-      <c r="AT14" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AT14">
+        <v>30</v>
       </c>
     </row>
     <row r="15">
@@ -2549,10 +2545,8 @@
           <t/>
         </is>
       </c>
-      <c r="AT15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AT15">
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -3151,10 +3145,8 @@
           <t/>
         </is>
       </c>
-      <c r="AT18" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AT18">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -3313,10 +3305,8 @@
           <t/>
         </is>
       </c>
-      <c r="AT19" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="AT19">
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -3458,7 +3448,7 @@
         <v>16</v>
       </c>
       <c r="AT20">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Atualização automática: 2026-08-25 04:26 UTC
</commit_message>
<xml_diff>
--- a/historico.xlsx
+++ b/historico.xlsx
@@ -308,6 +308,11 @@
           <t>24/08/2026</t>
         </is>
       </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -450,6 +455,9 @@
       <c r="AT2">
         <v>86</v>
       </c>
+      <c r="AU2">
+        <v>86</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -592,6 +600,9 @@
       <c r="AT3">
         <v>3</v>
       </c>
+      <c r="AU3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -734,6 +745,9 @@
       <c r="AT4">
         <v>1</v>
       </c>
+      <c r="AU4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -876,6 +890,9 @@
       <c r="AT5">
         <v>39</v>
       </c>
+      <c r="AU5">
+        <v>39</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1018,6 +1035,9 @@
       <c r="AT6">
         <v>33</v>
       </c>
+      <c r="AU6">
+        <v>33</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1232,6 +1252,11 @@
           <t/>
         </is>
       </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1428,6 +1453,11 @@
           <t/>
         </is>
       </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1606,6 +1636,9 @@
       <c r="AT9">
         <v>3</v>
       </c>
+      <c r="AU9">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1748,6 +1781,9 @@
       <c r="AT10">
         <v>7</v>
       </c>
+      <c r="AU10">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1890,6 +1926,9 @@
       <c r="AT11">
         <v>68</v>
       </c>
+      <c r="AU11">
+        <v>68</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2056,6 +2095,9 @@
       <c r="AT12">
         <v>3</v>
       </c>
+      <c r="AU12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2246,6 +2288,11 @@
           <t/>
         </is>
       </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2398,6 +2445,9 @@
       <c r="AT14">
         <v>30</v>
       </c>
+      <c r="AU14">
+        <v>30</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2548,6 +2598,9 @@
       <c r="AT15">
         <v>26</v>
       </c>
+      <c r="AU15">
+        <v>26</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2762,6 +2815,11 @@
           <t/>
         </is>
       </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2958,6 +3016,11 @@
           <t/>
         </is>
       </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3148,6 +3211,9 @@
       <c r="AT18">
         <v>3</v>
       </c>
+      <c r="AU18">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3308,6 +3374,9 @@
       <c r="AT19">
         <v>6</v>
       </c>
+      <c r="AU19">
+        <v>6</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3450,6 +3519,9 @@
       <c r="AT20">
         <v>18</v>
       </c>
+      <c r="AU20">
+        <v>18</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3590,6 +3662,9 @@
         <v>90</v>
       </c>
       <c r="AT21">
+        <v>90</v>
+      </c>
+      <c r="AU21">
         <v>90</v>
       </c>
     </row>

</xml_diff>